<commit_message>
Auto commit: 2026-09-05 22:11:20
</commit_message>
<xml_diff>
--- a/医药/康方/AK112_vs_K药_同适应症同期别配对分析.xlsx
+++ b/医药/康方/AK112_vs_K药_同适应症同期别配对分析.xlsx
@@ -21,6 +21,9 @@
     <sheet name="R3-两者均未成功" sheetId="12" state="visible" r:id="rId12"/>
     <sheet name="K药独占-AK112空白清单" sheetId="13" state="visible" r:id="rId13"/>
     <sheet name="反向速览矩阵" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="美国市场空间-配对适应症" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="美国市场空间-K药独占领域" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="美国测算口径与价格假设" sheetId="17" state="visible" r:id="rId17"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'配对总表'!$A$1:$O$16</definedName>
@@ -32,6 +35,8 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'R1-完全对等(K药胜)'!$A$1:$O$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'R2-头对头未证优效'!$A$1:$O$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'R3-两者均未成功'!$A$1:$O$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'美国市场空间-配对适应症'!$A$1:$P$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'美国市场空间-K药独占领域'!$A$1:$P$14</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -39,8 +44,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="9">
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="$#,##0"/>
+    <numFmt numFmtId="165" formatCode="#,##0.0"/>
+  </numFmts>
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -87,8 +95,13 @@
       <color rgb="00FFFFFF"/>
       <sz val="12"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="11">
+  <fills count="14">
     <fill>
       <patternFill/>
     </fill>
@@ -140,6 +153,21 @@
         <fgColor rgb="00F8CBAD"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DEEBF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F4CCCC"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -167,7 +195,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="66">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -291,6 +319,78 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="3" fontId="7" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="9" fontId="7" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -657,7 +757,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B34"/>
+  <dimension ref="A1:B43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1013,6 +1113,102 @@
       <c r="B34" s="4" t="inlineStr">
         <is>
           <t>同时满足三条：①早期研究已 COMPLETED；②完成后 12 个月以上不披露任何疗效数据；③不推进 III 期，且改用其他方案在同瘤种重启。符合者：AK112-207（HCC）、AK112-203（妇科）</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr"/>
+      <c r="B35" s="4" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="28" t="inlineStr">
+        <is>
+          <t>【2026-09-05 追加】美国市场空间测算</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>新增工作表</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>「美国市场空间-配对适应症」（21 条）、「美国市场空间-K药独占领域」（13 条）、「美国测算口径与价格假设」</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>地域口径</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>仅美国。发病数用 ACS《Cancer Statistics, 2026》Table 1 实测值；价格用 Merck 官方 WAC（2026-03）与 CMS Part B 净 ASP（J9271, Q3-2026）</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>价格双列</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>标价（WAC）年化 $213,299；实付（净 ASP）年化 $198,881。美国二者仅差约 7%，因 K药 走 Part B buy-and-bill 而非 PBM 回扣体系</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>双情景</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>天花板 = 全部符合条件患者 × 治疗时长 × 标价；现实情景 = 再乘治疗渗透率与竞争份额 × 治疗时长 × 实付净价</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>最关键的方法学点</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>空间 = 患者数 × **平均治疗时长** × 年费用。多数晚期适应症治疗不满一年（ES-SCLC 0.45 年、间皮瘤 0.35 年），漏掉这一项会系统性高估 30–60%</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>必须自行替换的变量</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>「现实情景可及患者」隐含的竞争份额假设（15%–45%，逐行标注）是全表最主观处，请按自己的判断替换后再使用</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>AK112 价格为占位值</t>
+        </is>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>Summit 从未披露美国定价，本表按与 K药 净价平价假设。注意依沃西 20mg/kg（70kg 患者 1,400mg/次）是 K药 200mg 的约 7 倍蛋白量，COGS 更高，构成定价下限约束</t>
         </is>
       </c>
     </row>
@@ -1125,7 +1321,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="30" t="n">
+      <c r="A2" s="43" t="n">
         <v>1</v>
       </c>
       <c r="B2" s="31" t="inlineStr">
@@ -1138,7 +1334,7 @@
           <t>★★★★★ 同瘤种/同线数/同期别/同方案（单药）</t>
         </is>
       </c>
-      <c r="D2" s="32" t="inlineStr">
+      <c r="D2" s="44" t="inlineStr">
         <is>
           <t>肝细胞癌（HCC）</t>
         </is>
@@ -1200,7 +1396,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="30" t="n">
+      <c r="A3" s="43" t="n">
         <v>2</v>
       </c>
       <c r="B3" s="31" t="inlineStr">
@@ -1213,7 +1409,7 @@
           <t>★★★★★ 同瘤种/同线数/同期别/同方案（单药）</t>
         </is>
       </c>
-      <c r="D3" s="32" t="inlineStr">
+      <c r="D3" s="44" t="inlineStr">
         <is>
           <t>宫颈癌</t>
         </is>
@@ -1275,7 +1471,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="30" t="n">
+      <c r="A4" s="43" t="n">
         <v>3</v>
       </c>
       <c r="B4" s="31" t="inlineStr">
@@ -1288,7 +1484,7 @@
           <t>★★★★☆ 同瘤种/同方案（单药），期别 II vs Ia/Ib+II</t>
         </is>
       </c>
-      <c r="D4" s="32" t="inlineStr">
+      <c r="D4" s="44" t="inlineStr">
         <is>
           <t>子宫内膜癌</t>
         </is>
@@ -1350,7 +1546,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="30" t="n">
+      <c r="A5" s="43" t="n">
         <v>4</v>
       </c>
       <c r="B5" s="31" t="inlineStr">
@@ -1363,7 +1559,7 @@
           <t>★★★☆☆ 同瘤种/同线数/同方案（单药），但 AK112 n=10 且剂量偏低</t>
         </is>
       </c>
-      <c r="D5" s="32" t="inlineStr">
+      <c r="D5" s="44" t="inlineStr">
         <is>
           <t>头颈鳞癌（HNSCC）</t>
         </is>
@@ -1534,7 +1730,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="30" t="n">
+      <c r="A2" s="43" t="n">
         <v>1</v>
       </c>
       <c r="B2" s="35" t="inlineStr">
@@ -1547,7 +1743,7 @@
           <t>★★★★☆ 同瘤种/同线数/同期别，且 K药 即为对照组</t>
         </is>
       </c>
-      <c r="D2" s="32" t="inlineStr">
+      <c r="D2" s="44" t="inlineStr">
         <is>
           <t>NSCLC（鳞）</t>
         </is>
@@ -1718,7 +1914,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="30" t="n">
+      <c r="A2" s="43" t="n">
         <v>1</v>
       </c>
       <c r="B2" s="36" t="inlineStr">
@@ -1731,7 +1927,7 @@
           <t>同瘤种/同线数/同期别/同方案 —— 但双方都失败</t>
         </is>
       </c>
-      <c r="D2" s="32" t="inlineStr">
+      <c r="D2" s="44" t="inlineStr">
         <is>
           <t>NSCLC（非鳞，EGFR 突变）</t>
         </is>
@@ -1793,7 +1989,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="30" t="n">
+      <c r="A3" s="43" t="n">
         <v>2</v>
       </c>
       <c r="B3" s="36" t="inlineStr">
@@ -1806,7 +2002,7 @@
           <t>同瘤种/同线数/同方案（单药）—— 双方均未获批</t>
         </is>
       </c>
-      <c r="D3" s="32" t="inlineStr">
+      <c r="D3" s="44" t="inlineStr">
         <is>
           <t>卵巢癌 / 输卵管 / 原发腹膜癌</t>
         </is>
@@ -1868,7 +2064,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="30" t="n">
+      <c r="A4" s="43" t="n">
         <v>3</v>
       </c>
       <c r="B4" s="36" t="inlineStr">
@@ -1881,7 +2077,7 @@
           <t>非疗效性失败，不可解读为阴性</t>
         </is>
       </c>
-      <c r="D4" s="32" t="inlineStr">
+      <c r="D4" s="44" t="inlineStr">
         <is>
           <t>卵巢癌</t>
         </is>
@@ -1943,7 +2139,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="30" t="n">
+      <c r="A5" s="43" t="n">
         <v>4</v>
       </c>
       <c r="B5" s="36" t="inlineStr">
@@ -1956,7 +2152,7 @@
           <t>同瘤种/同方案（单药）—— K药 更差</t>
         </is>
       </c>
-      <c r="D5" s="32" t="inlineStr">
+      <c r="D5" s="44" t="inlineStr">
         <is>
           <t>结直肠癌（MSS/pMMR）</t>
         </is>
@@ -2018,7 +2214,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="30" t="n">
+      <c r="A6" s="43" t="n">
         <v>5</v>
       </c>
       <c r="B6" s="36" t="inlineStr">
@@ -2031,7 +2227,7 @@
           <t>同瘤种/同方案（单药）—— K药 数据更完整但同样未获批</t>
         </is>
       </c>
-      <c r="D6" s="32" t="inlineStr">
+      <c r="D6" s="44" t="inlineStr">
         <is>
           <t>恶性胸膜间皮瘤</t>
         </is>
@@ -2093,7 +2289,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="30" t="n">
+      <c r="A7" s="43" t="n">
         <v>6</v>
       </c>
       <c r="B7" s="36" t="inlineStr">
@@ -2106,7 +2302,7 @@
           <t>同瘤种/同方案（单药）—— K药 数据更完整但同样未获批</t>
         </is>
       </c>
-      <c r="D7" s="32" t="inlineStr">
+      <c r="D7" s="44" t="inlineStr">
         <is>
           <t>肛管鳞癌</t>
         </is>
@@ -2823,6 +3019,2764 @@
           <t>非「AK112 失败」，是广度差距</t>
         </is>
       </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:P23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="66" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="9" customWidth="1" min="15" max="15"/>
+    <col width="68" customWidth="1" min="16" max="16"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="46" customHeight="1">
+      <c r="A1" s="42" t="inlineStr">
+        <is>
+          <t>序号</t>
+        </is>
+      </c>
+      <c r="B1" s="42" t="inlineStr">
+        <is>
+          <t>配对方向</t>
+        </is>
+      </c>
+      <c r="C1" s="42" t="inlineStr">
+        <is>
+          <t>瘤种</t>
+        </is>
+      </c>
+      <c r="D1" s="42" t="inlineStr">
+        <is>
+          <t>适应症 / 线数 / 设置</t>
+        </is>
+      </c>
+      <c r="E1" s="42" t="inlineStr">
+        <is>
+          <t>美国瘤种新发
+(ACS 2026)</t>
+        </is>
+      </c>
+      <c r="F1" s="42" t="inlineStr">
+        <is>
+          <t>美国现存患者
+(SEER 近似)</t>
+        </is>
+      </c>
+      <c r="G1" s="42" t="inlineStr">
+        <is>
+          <t>目标人群推算链（每步乘数已写明）</t>
+        </is>
+      </c>
+      <c r="H1" s="42" t="inlineStr">
+        <is>
+          <t>天花板
+可及患者</t>
+        </is>
+      </c>
+      <c r="I1" s="42" t="inlineStr">
+        <is>
+          <t>现实情景
+可及患者</t>
+        </is>
+      </c>
+      <c r="J1" s="42" t="inlineStr">
+        <is>
+          <t>平均治疗
+时长(年)</t>
+        </is>
+      </c>
+      <c r="K1" s="42" t="inlineStr">
+        <is>
+          <t>K药标价年化
+(WAC, US$)</t>
+        </is>
+      </c>
+      <c r="L1" s="42" t="inlineStr">
+        <is>
+          <t>K药实付年化
+(净ASP, US$)</t>
+        </is>
+      </c>
+      <c r="M1" s="42" t="inlineStr">
+        <is>
+          <t>天花板空间
+(百万US$/年, 标价)</t>
+        </is>
+      </c>
+      <c r="N1" s="42" t="inlineStr">
+        <is>
+          <t>现实情景空间
+(百万US$/年, 实付)</t>
+        </is>
+      </c>
+      <c r="O1" s="42" t="inlineStr">
+        <is>
+          <t>占比
+(现实/天花板)</t>
+        </is>
+      </c>
+      <c r="P1" s="42" t="inlineStr">
+        <is>
+          <t>关键假设与风险提示</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="43" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="11" t="inlineStr">
+        <is>
+          <t>AK112 胜 / K药 败</t>
+        </is>
+      </c>
+      <c r="C2" s="44" t="inlineStr">
+        <is>
+          <t>NSCLC（非鳞 EGFR 突变）</t>
+        </is>
+      </c>
+      <c r="D2" s="11" t="inlineStr">
+        <is>
+          <t>EGFR-TKI 进展后 二线 +培美曲塞/铂</t>
+        </is>
+      </c>
+      <c r="E2" s="45" t="n">
+        <v>229410</v>
+      </c>
+      <c r="F2" s="45" t="n">
+        <v>625000</v>
+      </c>
+      <c r="G2" s="11" t="inlineStr">
+        <is>
+          <t>肺癌 229,410 → NSCLC 85% = 195,000 → 非鳞 70% = 136,500 → EGFR 突变（美国人群）15% = 20,475 → 晚期/复发 70% = 14,333 → 一线 TKI 后进展并接受后线治疗 65% = 9,316</t>
+        </is>
+      </c>
+      <c r="H2" s="46" t="n">
+        <v>14333</v>
+      </c>
+      <c r="I2" s="47" t="n">
+        <v>4192</v>
+      </c>
+      <c r="J2" s="48" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="K2" s="49" t="n">
+        <v>213299.0476190476</v>
+      </c>
+      <c r="L2" s="49" t="n">
+        <v>198880.7277628032</v>
+      </c>
+      <c r="M2" s="50" t="n">
+        <v>1987.2</v>
+      </c>
+      <c r="N2" s="51" t="n">
+        <v>541.9</v>
+      </c>
+      <c r="O2" s="52" t="n">
+        <v>0.2727017703158223</v>
+      </c>
+      <c r="P2" s="11" t="inlineStr">
+        <is>
+          <t>现实情景按 AK112 获批后峰值份额 45% 假设（该线数目前无免疫标准，竞争少）。但 PDUFA 2026/11/14 存在延期风险，且 FDA 已表态需统计学显著 OS。美国 EGFR 突变率仅约 15%（亚洲约 40%），是该适应症在美国天然偏小的主因</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="43" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="11" t="inlineStr">
+        <is>
+          <t>口径有差异（AK112 III 期在做）</t>
+        </is>
+      </c>
+      <c r="C3" s="44" t="inlineStr">
+        <is>
+          <t>结直肠癌（MSS/pMMR）</t>
+        </is>
+      </c>
+      <c r="D3" s="11" t="inlineStr">
+        <is>
+          <t>一线转移性 +mFOLFOX</t>
+        </is>
+      </c>
+      <c r="E3" s="45" t="n">
+        <v>158850</v>
+      </c>
+      <c r="F3" s="45" t="n">
+        <v>1600000</v>
+      </c>
+      <c r="G3" s="11" t="inlineStr">
+        <is>
+          <t>CRC 158,850 → 转移性（初诊 IV 期 22% + 后续转移约 18%）40% = 63,540 → MSS/pMMR 95% = 60,363 → 接受一线系统治疗 80% = 48,290</t>
+        </is>
+      </c>
+      <c r="H3" s="46" t="n">
+        <v>60363</v>
+      </c>
+      <c r="I3" s="47" t="n">
+        <v>9658</v>
+      </c>
+      <c r="J3" s="48" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="K3" s="49" t="n">
+        <v>213299.0476190476</v>
+      </c>
+      <c r="L3" s="49" t="n">
+        <v>198880.7277628032</v>
+      </c>
+      <c r="M3" s="50" t="n">
+        <v>10300.3</v>
+      </c>
+      <c r="N3" s="51" t="n">
+        <v>1536.6</v>
+      </c>
+      <c r="O3" s="52" t="n">
+        <v>0.1491832861777865</v>
+      </c>
+      <c r="P3" s="11" t="inlineStr">
+        <is>
+          <t>全表第二大市场。但 K药 KEYNOTE-651 队列 B ORR 61% 已被判「与化疗相当」而放弃，CheckMate 9X8（nivo+化疗）随机试验亦失败。现实情景按 20% 份额，前提是 HARMONi-GI3（n=600）读出阳性——该赛道此前 0/N</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="43" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="11" t="inlineStr">
+        <is>
+          <t>口径有差异（K药 III 期该亚群已失败）</t>
+        </is>
+      </c>
+      <c r="C4" s="44" t="inlineStr">
+        <is>
+          <t>三阴性乳腺癌（TNBC）</t>
+        </is>
+      </c>
+      <c r="D4" s="11" t="inlineStr">
+        <is>
+          <t>一线转移性，PD-L1 CPS&lt;10 +紫杉类</t>
+        </is>
+      </c>
+      <c r="E4" s="45" t="n">
+        <v>324580</v>
+      </c>
+      <c r="F4" s="45" t="n">
+        <v>4300000</v>
+      </c>
+      <c r="G4" s="11" t="inlineStr">
+        <is>
+          <t>乳腺 324,580 → TNBC 12% = 38,950 → 转移性（初诊 IV 6% + 复发转移 24%）30% = 11,685 → CPS&lt;10 约 62% = 7,245 → 接受一线治疗 90% = 6,521</t>
+        </is>
+      </c>
+      <c r="H4" s="46" t="n">
+        <v>7245</v>
+      </c>
+      <c r="I4" s="47" t="n">
+        <v>1956</v>
+      </c>
+      <c r="J4" s="48" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="K4" s="49" t="n">
+        <v>213299.0476190476</v>
+      </c>
+      <c r="L4" s="49" t="n">
+        <v>198880.7277628032</v>
+      </c>
+      <c r="M4" s="50" t="n">
+        <v>1390.8</v>
+      </c>
+      <c r="N4" s="51" t="n">
+        <v>350.1</v>
+      </c>
+      <c r="O4" s="52" t="n">
+        <v>0.2517295763009811</v>
+      </c>
+      <c r="P4" s="11" t="inlineStr">
+        <is>
+          <t>这是 K药 在 III 期确证无获益的人群（KEYNOTE-355 的 CPS≥1 与 ITT 未达、KEYNOTE-119 全人群 OS 失败），因此若 HARMONi-BC1（n=416）成功即为增量市场。现实情景按 30% 份额。CPS&lt;10 占比按 KEYNOTE-355 分布外推</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="43" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t>双方均未成功</t>
+        </is>
+      </c>
+      <c r="C5" s="44" t="inlineStr">
+        <is>
+          <t>卵巢癌</t>
+        </is>
+      </c>
+      <c r="D5" s="11" t="inlineStr">
+        <is>
+          <t>铂耐药复发，单药</t>
+        </is>
+      </c>
+      <c r="E5" s="45" t="n">
+        <v>21010</v>
+      </c>
+      <c r="F5" s="45" t="n">
+        <v>250000</v>
+      </c>
+      <c r="G5" s="11" t="inlineStr">
+        <is>
+          <t>卵巢 21,010 → 晚期/复发并进入铂耐药 55% = 11,556 → 接受后线治疗 70% = 8,089</t>
+        </is>
+      </c>
+      <c r="H5" s="46" t="n">
+        <v>11556</v>
+      </c>
+      <c r="I5" s="47" t="n">
+        <v>809</v>
+      </c>
+      <c r="J5" s="48" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="K5" s="49" t="n">
+        <v>213299.0476190476</v>
+      </c>
+      <c r="L5" s="49" t="n">
+        <v>198880.7277628032</v>
+      </c>
+      <c r="M5" s="50" t="n">
+        <v>986</v>
+      </c>
+      <c r="N5" s="51" t="n">
+        <v>64.40000000000001</v>
+      </c>
+      <c r="O5" s="52" t="n">
+        <v>0.06527468318510837</v>
+      </c>
+      <c r="P5" s="11" t="inlineStr">
+        <is>
+          <t>K药 KEYNOTE-100（n=376）ORR 仅 8.0% 已否定，AK112 仅 Ia 期 n=19 且自己也放弃。现实情景按 10% 份额（几乎无路径），此格数字仅作理论参考，不应计入任何估值</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="43" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="11" t="inlineStr">
+        <is>
+          <t>双方均成功（AK112 头对头击败 K药）</t>
+        </is>
+      </c>
+      <c r="C6" s="44" t="inlineStr">
+        <is>
+          <t>NSCLC</t>
+        </is>
+      </c>
+      <c r="D6" s="11" t="inlineStr">
+        <is>
+          <t>一线 PD-L1 阳性（TPS≥1%）单药</t>
+        </is>
+      </c>
+      <c r="E6" s="45" t="n">
+        <v>229410</v>
+      </c>
+      <c r="F6" s="45" t="n">
+        <v>625000</v>
+      </c>
+      <c r="G6" s="11" t="inlineStr">
+        <is>
+          <t>肺癌 229,410 → NSCLC 85% = 195,000 → 晚期/转移 60% = 117,000 → 无驱动基因 75% = 87,750 → PD-L1 TPS≥1% 65% = 57,038 → 实际选择单药（不联化疗）约 35% = 19,963</t>
+        </is>
+      </c>
+      <c r="H6" s="46" t="n">
+        <v>57038</v>
+      </c>
+      <c r="I6" s="47" t="n">
+        <v>6987</v>
+      </c>
+      <c r="J6" s="48" t="n">
+        <v>1</v>
+      </c>
+      <c r="K6" s="49" t="n">
+        <v>213299.0476190476</v>
+      </c>
+      <c r="L6" s="49" t="n">
+        <v>198880.7277628032</v>
+      </c>
+      <c r="M6" s="50" t="n">
+        <v>12166.2</v>
+      </c>
+      <c r="N6" s="51" t="n">
+        <v>1389.6</v>
+      </c>
+      <c r="O6" s="52" t="n">
+        <v>0.1142168657909073</v>
+      </c>
+      <c r="P6" s="11" t="inlineStr">
+        <is>
+          <t>HARMONi-2 已 PFS+OS 双达标但全为中国人群，美国获批需 HARMONi-3 或新的全球试验支撑。天花板列按全部 TPS≥1% 晚期患者计（含目前联化疗者），若 AK112 单药能替代化免联合则天花板可及。现实情景按 35% 份额</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="43" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>双方均成功（未头对头）</t>
+        </is>
+      </c>
+      <c r="C7" s="44" t="inlineStr">
+        <is>
+          <t>NSCLC（鳞）</t>
+        </is>
+      </c>
+      <c r="D7" s="11" t="inlineStr">
+        <is>
+          <t>一线晚期 +含铂化疗</t>
+        </is>
+      </c>
+      <c r="E7" s="45" t="n">
+        <v>229410</v>
+      </c>
+      <c r="F7" s="45" t="n">
+        <v>625000</v>
+      </c>
+      <c r="G7" s="11" t="inlineStr">
+        <is>
+          <t>肺癌 229,410 → NSCLC 85% = 195,000 → 鳞癌 30% = 58,500 → 晚期/转移 60% = 35,100 → 接受一线系统治疗 85% = 29,835</t>
+        </is>
+      </c>
+      <c r="H7" s="46" t="n">
+        <v>35100</v>
+      </c>
+      <c r="I7" s="47" t="n">
+        <v>7459</v>
+      </c>
+      <c r="J7" s="48" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="K7" s="49" t="n">
+        <v>213299.0476190476</v>
+      </c>
+      <c r="L7" s="49" t="n">
+        <v>198880.7277628032</v>
+      </c>
+      <c r="M7" s="50" t="n">
+        <v>6738.1</v>
+      </c>
+      <c r="N7" s="51" t="n">
+        <v>1335.1</v>
+      </c>
+      <c r="O7" s="52" t="n">
+        <v>0.1981423342052539</v>
+      </c>
+      <c r="P7" s="11" t="inlineStr">
+        <is>
+          <t>HARMONi-6 OS HR 0.66 但对照为替雷利珠+化疗（美国未上市），无法直接支撑美国注册。美国注册须靠 HARMONi-3 鳞癌队列（vs K药+化疗），而该队列期中 PFS 已未达界值</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="43" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>双方均成功（对照强度不同）</t>
+        </is>
+      </c>
+      <c r="C8" s="44" t="inlineStr">
+        <is>
+          <t>胆道癌（BTC）</t>
+        </is>
+      </c>
+      <c r="D8" s="11" t="inlineStr">
+        <is>
+          <t>一线不可切除 +吉西他滨/顺铂</t>
+        </is>
+      </c>
+      <c r="E8" s="45" t="n">
+        <v>19000</v>
+      </c>
+      <c r="F8" s="45" t="n">
+        <v>35000</v>
+      </c>
+      <c r="G8" s="11" t="inlineStr">
+        <is>
+          <t>胆囊及其他胆道 12,640 + 肝内胆管（含于 liver&amp;IBD 42,340 中约 15% = 6,351）≈ 19,000 → 晚期/不可切除 70% = 13,300 → 接受一线系统治疗 75% = 9,975</t>
+        </is>
+      </c>
+      <c r="H8" s="46" t="n">
+        <v>13300</v>
+      </c>
+      <c r="I8" s="47" t="n">
+        <v>2993</v>
+      </c>
+      <c r="J8" s="48" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="K8" s="49" t="n">
+        <v>213299.0476190476</v>
+      </c>
+      <c r="L8" s="49" t="n">
+        <v>198880.7277628032</v>
+      </c>
+      <c r="M8" s="50" t="n">
+        <v>1985.8</v>
+      </c>
+      <c r="N8" s="51" t="n">
+        <v>416.7</v>
+      </c>
+      <c r="O8" s="52" t="n">
+        <v>0.2098257866844918</v>
+      </c>
+      <c r="P8" s="11" t="inlineStr">
+        <is>
+          <t>HARMONi-GI1 头对头击败度伐利尤+化疗（OS 显著），但 HR 与中位数至今未披露，无法核验。K药 KEYNOTE-966 已获批（OS HR 0.83）。现实情景按 30% 份额。该瘤种美国发病数小，是典型「机制验证价值 &gt; 商业价值」的适应症</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="43" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="11" t="inlineStr">
+        <is>
+          <t>K药 已成功（AK112 仅 II 期单臂）</t>
+        </is>
+      </c>
+      <c r="C9" s="44" t="inlineStr">
+        <is>
+          <t>NSCLC</t>
+        </is>
+      </c>
+      <c r="D9" s="11" t="inlineStr">
+        <is>
+          <t>可切除 II–IIIB 期 围手术期</t>
+        </is>
+      </c>
+      <c r="E9" s="45" t="n">
+        <v>229410</v>
+      </c>
+      <c r="F9" s="45" t="n">
+        <v>625000</v>
+      </c>
+      <c r="G9" s="11" t="inlineStr">
+        <is>
+          <t>肺癌 229,410 → NSCLC 85% = 195,000 → 可切除 II–IIIB(N2) 期约 20% = 39,000 → 接受新辅助免疫治疗 60% = 23,400</t>
+        </is>
+      </c>
+      <c r="H9" s="46" t="n">
+        <v>39000</v>
+      </c>
+      <c r="I9" s="47" t="n">
+        <v>4680</v>
+      </c>
+      <c r="J9" s="48" t="n">
+        <v>1</v>
+      </c>
+      <c r="K9" s="49" t="n">
+        <v>213299.0476190476</v>
+      </c>
+      <c r="L9" s="49" t="n">
+        <v>198880.7277628032</v>
+      </c>
+      <c r="M9" s="50" t="n">
+        <v>8318.700000000001</v>
+      </c>
+      <c r="N9" s="51" t="n">
+        <v>930.8</v>
+      </c>
+      <c r="O9" s="52" t="n">
+        <v>0.1118883914294851</v>
+      </c>
+      <c r="P9" s="11" t="inlineStr">
+        <is>
+          <t>K药 KEYNOTE-671 已获批（EFS HR 0.58 / OS HR 0.72）。AK112 仅 60 例 II 期单臂、EFS 未成熟、无 III 期，短期无法进入。现实情景按 20% 份额，实为长期期权而非在手资产</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="43" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="11" t="inlineStr">
+        <is>
+          <t>K药 已成功（AK112 仅单中心 IIT）</t>
+        </is>
+      </c>
+      <c r="C10" s="44" t="inlineStr">
+        <is>
+          <t>头颈鳞癌（HNSCC）</t>
+        </is>
+      </c>
+      <c r="D10" s="11" t="inlineStr">
+        <is>
+          <t>可切除局部晚期 围手术期（CPS≥1）</t>
+        </is>
+      </c>
+      <c r="E10" s="45" t="n">
+        <v>72770</v>
+      </c>
+      <c r="F10" s="45" t="n">
+        <v>490000</v>
+      </c>
+      <c r="G10" s="11" t="inlineStr">
+        <is>
+          <t>口腔咽 60,480 + 喉 12,290 = 72,770 → 鳞癌 90% = 65,493 → 可切除局晚 III–IVA 期 35% = 22,923 → CPS≥1 约 85% = 19,484 → 接受围手术期治疗 55% = 10,716</t>
+        </is>
+      </c>
+      <c r="H10" s="46" t="n">
+        <v>19484</v>
+      </c>
+      <c r="I10" s="47" t="n">
+        <v>1607</v>
+      </c>
+      <c r="J10" s="48" t="n">
+        <v>1</v>
+      </c>
+      <c r="K10" s="49" t="n">
+        <v>213299.0476190476</v>
+      </c>
+      <c r="L10" s="49" t="n">
+        <v>198880.7277628032</v>
+      </c>
+      <c r="M10" s="50" t="n">
+        <v>4155.9</v>
+      </c>
+      <c r="N10" s="51" t="n">
+        <v>319.6</v>
+      </c>
+      <c r="O10" s="52" t="n">
+        <v>0.07690269153629585</v>
+      </c>
+      <c r="P10" s="11" t="inlineStr">
+        <is>
+          <t>K药 KEYNOTE-689 2025/6 已获批（EFS HR 0.70）。AK112 仅 36 例单中心 IIT，且喉部原发 pCR 仅 12.5% 是明显短板。现实情景按 15% 份额</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="43" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="11" t="inlineStr">
+        <is>
+          <t>K药 已成功（同期别 ORR 差距有限）</t>
+        </is>
+      </c>
+      <c r="C11" s="44" t="inlineStr">
+        <is>
+          <t>胃 / 胃食管结合部腺癌</t>
+        </is>
+      </c>
+      <c r="D11" s="11" t="inlineStr">
+        <is>
+          <t>一线晚期 +化疗（HER2 阴性）</t>
+        </is>
+      </c>
+      <c r="E11" s="45" t="n">
+        <v>38270</v>
+      </c>
+      <c r="F11" s="45" t="n">
+        <v>130000</v>
+      </c>
+      <c r="G11" s="11" t="inlineStr">
+        <is>
+          <t>胃 31,510 + GEJ（含于食管 22,530 中约 30% = 6,759）≈ 38,270 → 晚期/转移 60% = 22,962 → HER2 阴性 80% = 18,370 → 接受一线治疗 80% = 14,696</t>
+        </is>
+      </c>
+      <c r="H11" s="46" t="n">
+        <v>22962</v>
+      </c>
+      <c r="I11" s="47" t="n">
+        <v>2204</v>
+      </c>
+      <c r="J11" s="48" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="K11" s="49" t="n">
+        <v>213299.0476190476</v>
+      </c>
+      <c r="L11" s="49" t="n">
+        <v>198880.7277628032</v>
+      </c>
+      <c r="M11" s="50" t="n">
+        <v>3428.4</v>
+      </c>
+      <c r="N11" s="51" t="n">
+        <v>306.8</v>
+      </c>
+      <c r="O11" s="52" t="n">
+        <v>0.08949641970450645</v>
+      </c>
+      <c r="P11" s="11" t="inlineStr">
+        <is>
+          <t>K药 KEYNOTE-859（OS HR 0.78）与 KEYNOTE-811（HER2+）均已获批。AK112 的 ORR 71.7% 需叠加卡度尼利（AK104），是四药方案，成本与毒性口径完全不同，且无胃癌 III 期。现实情景按 15% 份额</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="43" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="11" t="inlineStr">
+        <is>
+          <t>K药 机制不适用（AK112 独占场景）</t>
+        </is>
+      </c>
+      <c r="C12" s="44" t="inlineStr">
+        <is>
+          <t>NSCLC</t>
+        </is>
+      </c>
+      <c r="D12" s="11" t="inlineStr">
+        <is>
+          <t>PD-(L)1 经治 / IO 耐药后 +多西他赛</t>
+        </is>
+      </c>
+      <c r="E12" s="45" t="n">
+        <v>229410</v>
+      </c>
+      <c r="F12" s="45" t="n">
+        <v>625000</v>
+      </c>
+      <c r="G12" s="11" t="inlineStr">
+        <is>
+          <t>肺癌 229,410 → NSCLC 85% = 195,000 → 晚期并接受过一线免疫治疗 55% = 107,250 → 进展后接受二线治疗 50% = 53,625</t>
+        </is>
+      </c>
+      <c r="H12" s="46" t="n">
+        <v>53625</v>
+      </c>
+      <c r="I12" s="47" t="n">
+        <v>8044</v>
+      </c>
+      <c r="J12" s="48" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="K12" s="49" t="n">
+        <v>213299.0476190476</v>
+      </c>
+      <c r="L12" s="49" t="n">
+        <v>198880.7277628032</v>
+      </c>
+      <c r="M12" s="50" t="n">
+        <v>6862.9</v>
+      </c>
+      <c r="N12" s="51" t="n">
+        <v>959.9</v>
+      </c>
+      <c r="O12" s="52" t="n">
+        <v>0.1398648361552103</v>
+      </c>
+      <c r="P12" s="11" t="inlineStr">
+        <is>
+          <t>全表第三大市场，且 K药 机制上无法进入（它自身即耐药来源）。这是 AK112 最干净的差异化场景。但目前仅 AK112-201 的 n=20 数据，III 期 HARMONi-8A（n=536）尚无读出。现实情景按 15% 份额</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="43" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="11" t="inlineStr">
+        <is>
+          <t>K药 完败（AK112 数据未公开）</t>
+        </is>
+      </c>
+      <c r="C13" s="44" t="inlineStr">
+        <is>
+          <t>胰腺癌（PDAC）</t>
+        </is>
+      </c>
+      <c r="D13" s="11" t="inlineStr">
+        <is>
+          <t>一线转移性 +吉西他滨/白蛋白紫杉醇</t>
+        </is>
+      </c>
+      <c r="E13" s="45" t="n">
+        <v>67530</v>
+      </c>
+      <c r="F13" s="45" t="n">
+        <v>65000</v>
+      </c>
+      <c r="G13" s="11" t="inlineStr">
+        <is>
+          <t>胰腺 67,530 → 转移性 52% = 35,116 → 接受一线化疗 65% = 22,825</t>
+        </is>
+      </c>
+      <c r="H13" s="46" t="n">
+        <v>35116</v>
+      </c>
+      <c r="I13" s="47" t="n">
+        <v>1826</v>
+      </c>
+      <c r="J13" s="48" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="K13" s="49" t="n">
+        <v>213299.0476190476</v>
+      </c>
+      <c r="L13" s="49" t="n">
+        <v>198880.7277628032</v>
+      </c>
+      <c r="M13" s="50" t="n">
+        <v>3745.1</v>
+      </c>
+      <c r="N13" s="51" t="n">
+        <v>181.6</v>
+      </c>
+      <c r="O13" s="52" t="n">
+        <v>0.04848411995250024</v>
+      </c>
+      <c r="P13" s="11" t="inlineStr">
+        <is>
+          <t>K药 KEYNOTE-028 ORR 0%（全项目最差）。AK112-210 的 II 期数据至今未公开，999 例 III 期（HARMONi-GI2）只是开发决策而非数据证据。现实情景按 8% 份额（极低成功概率），此格不应计入任何近期估值</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="43" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="11" t="inlineStr">
+        <is>
+          <t>K药 III 期失败（AK112 未验证）</t>
+        </is>
+      </c>
+      <c r="C14" s="44" t="inlineStr">
+        <is>
+          <t>小细胞肺癌（SCLC）</t>
+        </is>
+      </c>
+      <c r="D14" s="11" t="inlineStr">
+        <is>
+          <t>一线广泛期 +依托泊苷/铂</t>
+        </is>
+      </c>
+      <c r="E14" s="45" t="n">
+        <v>29820</v>
+      </c>
+      <c r="F14" s="45" t="n">
+        <v>625000</v>
+      </c>
+      <c r="G14" s="11" t="inlineStr">
+        <is>
+          <t>肺癌 229,410 → SCLC 13% = 29,823 → 广泛期 70% = 20,876 → 接受一线治疗 80% = 16,701</t>
+        </is>
+      </c>
+      <c r="H14" s="46" t="n">
+        <v>20876</v>
+      </c>
+      <c r="I14" s="47" t="n">
+        <v>2505</v>
+      </c>
+      <c r="J14" s="48" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="K14" s="49" t="n">
+        <v>213299.0476190476</v>
+      </c>
+      <c r="L14" s="49" t="n">
+        <v>198880.7277628032</v>
+      </c>
+      <c r="M14" s="50" t="n">
+        <v>2003.8</v>
+      </c>
+      <c r="N14" s="51" t="n">
+        <v>224.2</v>
+      </c>
+      <c r="O14" s="52" t="n">
+        <v>0.1118830317632929</v>
+      </c>
+      <c r="P14" s="11" t="inlineStr">
+        <is>
+          <t>K药 KEYNOTE-604 OS 未达（HR 0.80, p=0.0164），SCLC 三线适应症已撤回。AK112 仅 Ib 期 ORR 87.5% 但 mPFS 6.9 月增量有限，至今未开 1L III 期。治疗时长短（0.45 年）严重压缩商业价值</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="43" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="11" t="inlineStr">
+        <is>
+          <t>K药 胜 / AK112 隐性失败</t>
+        </is>
+      </c>
+      <c r="C15" s="44" t="inlineStr">
+        <is>
+          <t>肝细胞癌（HCC）</t>
+        </is>
+      </c>
+      <c r="D15" s="11" t="inlineStr">
+        <is>
+          <t>系统治疗后 二线（及一线联合）</t>
+        </is>
+      </c>
+      <c r="E15" s="45" t="n">
+        <v>33870</v>
+      </c>
+      <c r="F15" s="45" t="n">
+        <v>70000</v>
+      </c>
+      <c r="G15" s="11" t="inlineStr">
+        <is>
+          <t>liver &amp; IBD 42,340 → HCC 约 80% = 33,872 → 晚期/不可切除 60% = 20,323 → 接受一线系统治疗 70% = 14,226 → 进展后接受二线 55% = 7,824</t>
+        </is>
+      </c>
+      <c r="H15" s="46" t="n">
+        <v>20323</v>
+      </c>
+      <c r="I15" s="47" t="n">
+        <v>1565</v>
+      </c>
+      <c r="J15" s="48" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="K15" s="49" t="n">
+        <v>213299.0476190476</v>
+      </c>
+      <c r="L15" s="49" t="n">
+        <v>198880.7277628032</v>
+      </c>
+      <c r="M15" s="50" t="n">
+        <v>2167.4</v>
+      </c>
+      <c r="N15" s="51" t="n">
+        <v>155.6</v>
+      </c>
+      <c r="O15" s="52" t="n">
+        <v>0.07180096958583224</v>
+      </c>
+      <c r="P15" s="11" t="inlineStr">
+        <is>
+          <t>K药 KEYNOTE-224 ORR 17% 加速批准 + KEYNOTE-394 OS HR 0.79 转完全批准（但全球 KEYNOTE-240 曾失败）。AK112-207 完成后不披露数据、无 III 期，已换 AK112-209（+AK130 / +AK127 / +卡度尼利，并加信迪利+贝伐对照臂）重启。现实情景按 20% 份额</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="43" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="11" t="inlineStr">
+        <is>
+          <t>K药 胜 / AK112 隐性失败</t>
+        </is>
+      </c>
+      <c r="C16" s="44" t="inlineStr">
+        <is>
+          <t>宫颈癌</t>
+        </is>
+      </c>
+      <c r="D16" s="11" t="inlineStr">
+        <is>
+          <t>既往化疗失败 二线 单药</t>
+        </is>
+      </c>
+      <c r="E16" s="45" t="n">
+        <v>13490</v>
+      </c>
+      <c r="F16" s="45" t="n">
+        <v>290000</v>
+      </c>
+      <c r="G16" s="11" t="inlineStr">
+        <is>
+          <t>宫颈 13,490 → 复发/转移 35% = 4,722 → CPS≥1 约 85% = 4,013 → 接受二线治疗 70% = 2,809</t>
+        </is>
+      </c>
+      <c r="H16" s="46" t="n">
+        <v>4722</v>
+      </c>
+      <c r="I16" s="47" t="n">
+        <v>702</v>
+      </c>
+      <c r="J16" s="48" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="K16" s="49" t="n">
+        <v>213299.0476190476</v>
+      </c>
+      <c r="L16" s="49" t="n">
+        <v>198880.7277628032</v>
+      </c>
+      <c r="M16" s="50" t="n">
+        <v>402.9</v>
+      </c>
+      <c r="N16" s="51" t="n">
+        <v>55.8</v>
+      </c>
+      <c r="O16" s="52" t="n">
+        <v>0.138616495100061</v>
+      </c>
+      <c r="P16" s="11" t="inlineStr">
+        <is>
+          <t>K药 该二线单药加速批准已于 2024 撤回（被自家一线 KEYNOTE-826 取代，非疗效失败）。宫颈癌真正的大空间在一线（OS HR 0.60）与局晚同步放化疗（OS HR 0.67），AK112 在这两个场景亦无数据。AK112-203 完成后不披露，康方自己 0 项后继研究</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="43" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="11" t="inlineStr">
+        <is>
+          <t>K药 胜 / AK112 未成队列</t>
+        </is>
+      </c>
+      <c r="C17" s="44" t="inlineStr">
+        <is>
+          <t>子宫内膜癌</t>
+        </is>
+      </c>
+      <c r="D17" s="11" t="inlineStr">
+        <is>
+          <t>既往治疗失败 二线（dMMR 单药 / pMMR 联合）</t>
+        </is>
+      </c>
+      <c r="E17" s="45" t="n">
+        <v>68270</v>
+      </c>
+      <c r="F17" s="45" t="n">
+        <v>920000</v>
+      </c>
+      <c r="G17" s="11" t="inlineStr">
+        <is>
+          <t>子宫体 68,270 → 晚期/复发 25% = 17,068 → dMMR 亚群 27.5% = 4,694 → 接受二线治疗 75% = 3,520</t>
+        </is>
+      </c>
+      <c r="H17" s="46" t="n">
+        <v>17068</v>
+      </c>
+      <c r="I17" s="47" t="n">
+        <v>1408</v>
+      </c>
+      <c r="J17" s="48" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="K17" s="49" t="n">
+        <v>213299.0476190476</v>
+      </c>
+      <c r="L17" s="49" t="n">
+        <v>198880.7277628032</v>
+      </c>
+      <c r="M17" s="50" t="n">
+        <v>4368.7</v>
+      </c>
+      <c r="N17" s="51" t="n">
+        <v>336</v>
+      </c>
+      <c r="O17" s="52" t="n">
+        <v>0.07691725994683769</v>
+      </c>
+      <c r="P17" s="11" t="inlineStr">
+        <is>
+          <t>K药 dMMR 富集后 ORR 48–50% 获批，pMMR 靠 +lenvatinib（OS HR 0.68）获批，一线 NRG-GY018 dMMR PFS HR 0.30。AK112 从未做 dMMR 富集队列——这是研发策略缺失而非药物更弱（K药 未富集时 ORR 也只有 13%）。治疗时长 1.2 年（dMMR 应答极持久）</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="43" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="11" t="inlineStr">
+        <is>
+          <t>K药 胜 / AK112 路线废弃</t>
+        </is>
+      </c>
+      <c r="C18" s="44" t="inlineStr">
+        <is>
+          <t>头颈鳞癌（HNSCC）</t>
+        </is>
+      </c>
+      <c r="D18" s="11" t="inlineStr">
+        <is>
+          <t>一线复发/转移 单药（CPS≥1）</t>
+        </is>
+      </c>
+      <c r="E18" s="45" t="n">
+        <v>72770</v>
+      </c>
+      <c r="F18" s="45" t="n">
+        <v>490000</v>
+      </c>
+      <c r="G18" s="11" t="inlineStr">
+        <is>
+          <t>HNSCC 65,493 → 复发/转移 30% = 19,648 → CPS≥1 约 85% = 16,701 → 实际选择单药（CPS≥20 或不耐化疗）约 40% = 6,680</t>
+        </is>
+      </c>
+      <c r="H18" s="46" t="n">
+        <v>19648</v>
+      </c>
+      <c r="I18" s="47" t="n">
+        <v>2004</v>
+      </c>
+      <c r="J18" s="48" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="K18" s="49" t="n">
+        <v>213299.0476190476</v>
+      </c>
+      <c r="L18" s="49" t="n">
+        <v>198880.7277628032</v>
+      </c>
+      <c r="M18" s="50" t="n">
+        <v>2933.6</v>
+      </c>
+      <c r="N18" s="51" t="n">
+        <v>279</v>
+      </c>
+      <c r="O18" s="52" t="n">
+        <v>0.09510057699879897</v>
+      </c>
+      <c r="P18" s="11" t="inlineStr">
+        <is>
+          <t>K药 KEYNOTE-012 ORR 18% → KEYNOTE-048 CPS≥20 OS HR 0.61 已成一线标准。AK112 单药 n=10 且 CPS≥20 亚组 ORR 0%（与 K药 方向性相反），路线废弃改走联合。但剂量仅 10mg/kg，可能低估</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="43" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="11" t="inlineStr">
+        <is>
+          <t>AK112 头对头未证优效（未定论）</t>
+        </is>
+      </c>
+      <c r="C19" s="44" t="inlineStr">
+        <is>
+          <t>NSCLC（非鳞）</t>
+        </is>
+      </c>
+      <c r="D19" s="11" t="inlineStr">
+        <is>
+          <t>一线晚期 +培美曲塞/铂（vs K药+化疗）</t>
+        </is>
+      </c>
+      <c r="E19" s="45" t="n">
+        <v>229410</v>
+      </c>
+      <c r="F19" s="45" t="n">
+        <v>625000</v>
+      </c>
+      <c r="G19" s="11" t="inlineStr">
+        <is>
+          <t>肺癌 229,410 → NSCLC 85% = 195,000 → 非鳞 70% = 136,500 → 晚期/转移 60% = 81,900 → 无驱动基因 70% = 57,330 → 接受一线化免联合 85% = 48,731</t>
+        </is>
+      </c>
+      <c r="H19" s="46" t="n">
+        <v>57330</v>
+      </c>
+      <c r="I19" s="47" t="n">
+        <v>9746</v>
+      </c>
+      <c r="J19" s="48" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="K19" s="49" t="n">
+        <v>213299.0476190476</v>
+      </c>
+      <c r="L19" s="49" t="n">
+        <v>198880.7277628032</v>
+      </c>
+      <c r="M19" s="50" t="n">
+        <v>10394.2</v>
+      </c>
+      <c r="N19" s="51" t="n">
+        <v>1647.5</v>
+      </c>
+      <c r="O19" s="52" t="n">
+        <v>0.1585069281457879</v>
+      </c>
+      <c r="P19" s="11" t="inlineStr">
+        <is>
+          <t>**全表最大单一市场**，也是 HARMONi-3 非鳞队列（2027 H1 读出 PFS）的标的。K药 KEYNOTE-189 OS HR 0.56 是全项目最强效应量之一，是极高的对照门槛。鳞癌队列期中 PFS 已未达界值。现实情景按 20% 份额</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="43" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="11" t="inlineStr">
+        <is>
+          <t>双方均未成功</t>
+        </is>
+      </c>
+      <c r="C20" s="44" t="inlineStr">
+        <is>
+          <t>恶性胸膜间皮瘤</t>
+        </is>
+      </c>
+      <c r="D20" s="11" t="inlineStr">
+        <is>
+          <t>既往治疗过，单药</t>
+        </is>
+      </c>
+      <c r="E20" s="45" t="n">
+        <v>3000</v>
+      </c>
+      <c r="F20" s="45" t="n">
+        <v>4000</v>
+      </c>
+      <c r="G20" s="11" t="inlineStr">
+        <is>
+          <t>间皮瘤约 3,000（含于 other respiratory organs 6,120）→ 不可切除/经治 80% = 2,400 → 接受二线治疗 60% = 1,440</t>
+        </is>
+      </c>
+      <c r="H20" s="46" t="n">
+        <v>2400</v>
+      </c>
+      <c r="I20" s="47" t="n">
+        <v>216</v>
+      </c>
+      <c r="J20" s="48" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="K20" s="49" t="n">
+        <v>213299.0476190476</v>
+      </c>
+      <c r="L20" s="49" t="n">
+        <v>198880.7277628032</v>
+      </c>
+      <c r="M20" s="50" t="n">
+        <v>179.2</v>
+      </c>
+      <c r="N20" s="51" t="n">
+        <v>15</v>
+      </c>
+      <c r="O20" s="52" t="n">
+        <v>0.08391629357211385</v>
+      </c>
+      <c r="P20" s="11" t="inlineStr">
+        <is>
+          <t>K药 KEYNOTE-158 ORR 8.0%、DOR 14.3 月但 III 期 PROMISE-meso 失败、未获批；AK112 仅个别 PR。发病数极小 + 治疗时长极短，商业价值可忽略</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="43" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="11" t="inlineStr">
+        <is>
+          <t>双方均未成功</t>
+        </is>
+      </c>
+      <c r="C21" s="44" t="inlineStr">
+        <is>
+          <t>肛管鳞癌</t>
+        </is>
+      </c>
+      <c r="D21" s="11" t="inlineStr">
+        <is>
+          <t>既往治疗过，单药</t>
+        </is>
+      </c>
+      <c r="E21" s="45" t="n">
+        <v>11270</v>
+      </c>
+      <c r="F21" s="45" t="n">
+        <v>40000</v>
+      </c>
+      <c r="G21" s="11" t="inlineStr">
+        <is>
+          <t>肛管 11,270 → 鳞癌 85% = 9,580 → 复发/转移 20% = 1,916 → 接受二线治疗 65% = 1,245</t>
+        </is>
+      </c>
+      <c r="H21" s="46" t="n">
+        <v>1916</v>
+      </c>
+      <c r="I21" s="47" t="n">
+        <v>249</v>
+      </c>
+      <c r="J21" s="48" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="K21" s="49" t="n">
+        <v>213299.0476190476</v>
+      </c>
+      <c r="L21" s="49" t="n">
+        <v>198880.7277628032</v>
+      </c>
+      <c r="M21" s="50" t="n">
+        <v>163.5</v>
+      </c>
+      <c r="N21" s="51" t="n">
+        <v>19.8</v>
+      </c>
+      <c r="O21" s="52" t="n">
+        <v>0.1211734928059403</v>
+      </c>
+      <c r="P21" s="11" t="inlineStr">
+        <is>
+          <t>K药 KEYNOTE-158 队列 A ORR 11%（n=112）未获批；AK112 仅个别 PR。商业价值可忽略</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="43" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="11" t="inlineStr">
+        <is>
+          <t>技术上不可及（现实情景为 0）</t>
+        </is>
+      </c>
+      <c r="C22" s="44" t="inlineStr">
+        <is>
+          <t>结直肠癌（MSS/pMMR）</t>
+        </is>
+      </c>
+      <c r="D22" s="11" t="inlineStr">
+        <is>
+          <t>晚期经治 单药</t>
+        </is>
+      </c>
+      <c r="E22" s="45" t="n">
+        <v>158850</v>
+      </c>
+      <c r="F22" s="45" t="n">
+        <v>1600000</v>
+      </c>
+      <c r="G22" s="11" t="inlineStr">
+        <is>
+          <t>同一线 MSS mCRC 池：60,363 例 → 但 K药 单药 ORR 0–4%、AK112 单药仅个别 PR</t>
+        </is>
+      </c>
+      <c r="H22" s="46" t="n">
+        <v>60363</v>
+      </c>
+      <c r="I22" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="J22" s="48" t="n">
+        <v>0</v>
+      </c>
+      <c r="K22" s="49" t="n">
+        <v>213299.0476190476</v>
+      </c>
+      <c r="L22" s="49" t="n">
+        <v>198880.7277628032</v>
+      </c>
+      <c r="M22" s="50" t="n">
+        <v>0</v>
+      </c>
+      <c r="N22" s="54" t="n">
+        <v>0</v>
+      </c>
+      <c r="O22" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="P22" s="11" t="inlineStr">
+        <is>
+          <t>刻意保留此行并把现实情景设为 0：这是 PD-1 单药在 MSS CRC 的确证性失败区，说明「天花板大」与「可及」是两件事。任何按天花板估值的模型都会在这类行上出错</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="55" t="n"/>
+      <c r="B23" s="56" t="inlineStr">
+        <is>
+          <t>合计</t>
+        </is>
+      </c>
+      <c r="C23" s="57" t="n"/>
+      <c r="D23" s="56" t="n"/>
+      <c r="E23" s="58" t="n"/>
+      <c r="F23" s="58" t="n"/>
+      <c r="G23" s="56" t="inlineStr">
+        <is>
+          <t>注：合计仅供量级校准；同一瘤种不同线数存在患者池重叠，不可简单相加</t>
+        </is>
+      </c>
+      <c r="H23" s="58" t="n"/>
+      <c r="I23" s="58" t="n"/>
+      <c r="J23" s="59" t="n"/>
+      <c r="K23" s="60" t="n"/>
+      <c r="L23" s="60" t="n"/>
+      <c r="M23" s="61" t="n">
+        <v>84678.60000000001</v>
+      </c>
+      <c r="N23" s="61" t="n">
+        <v>11066.1</v>
+      </c>
+      <c r="O23" s="62" t="n">
+        <v>0.1306834471711254</v>
+      </c>
+      <c r="P23" s="56" t="n"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:P22"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:P15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="66" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="9" customWidth="1" min="15" max="15"/>
+    <col width="68" customWidth="1" min="16" max="16"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="46" customHeight="1">
+      <c r="A1" s="42" t="inlineStr">
+        <is>
+          <t>序号</t>
+        </is>
+      </c>
+      <c r="B1" s="42" t="inlineStr">
+        <is>
+          <t>配对方向</t>
+        </is>
+      </c>
+      <c r="C1" s="42" t="inlineStr">
+        <is>
+          <t>瘤种</t>
+        </is>
+      </c>
+      <c r="D1" s="42" t="inlineStr">
+        <is>
+          <t>适应症 / 线数 / 设置</t>
+        </is>
+      </c>
+      <c r="E1" s="42" t="inlineStr">
+        <is>
+          <t>美国瘤种新发
+(ACS 2026)</t>
+        </is>
+      </c>
+      <c r="F1" s="42" t="inlineStr">
+        <is>
+          <t>美国现存患者
+(SEER 近似)</t>
+        </is>
+      </c>
+      <c r="G1" s="42" t="inlineStr">
+        <is>
+          <t>目标人群推算链（每步乘数已写明）</t>
+        </is>
+      </c>
+      <c r="H1" s="42" t="inlineStr">
+        <is>
+          <t>天花板
+可及患者</t>
+        </is>
+      </c>
+      <c r="I1" s="42" t="inlineStr">
+        <is>
+          <t>现实情景
+可及患者</t>
+        </is>
+      </c>
+      <c r="J1" s="42" t="inlineStr">
+        <is>
+          <t>平均治疗
+时长(年)</t>
+        </is>
+      </c>
+      <c r="K1" s="42" t="inlineStr">
+        <is>
+          <t>K药标价年化
+(WAC, US$)</t>
+        </is>
+      </c>
+      <c r="L1" s="42" t="inlineStr">
+        <is>
+          <t>K药实付年化
+(净ASP, US$)</t>
+        </is>
+      </c>
+      <c r="M1" s="42" t="inlineStr">
+        <is>
+          <t>天花板空间
+(百万US$/年, 标价)</t>
+        </is>
+      </c>
+      <c r="N1" s="42" t="inlineStr">
+        <is>
+          <t>现实情景空间
+(百万US$/年, 实付)</t>
+        </is>
+      </c>
+      <c r="O1" s="42" t="inlineStr">
+        <is>
+          <t>占比
+(现实/天花板)</t>
+        </is>
+      </c>
+      <c r="P1" s="42" t="inlineStr">
+        <is>
+          <t>关键假设与风险提示</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="43" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="11" t="inlineStr">
+        <is>
+          <t>K药 独占（AK112 空白）</t>
+        </is>
+      </c>
+      <c r="C2" s="44" t="inlineStr">
+        <is>
+          <t>黑色素瘤</t>
+        </is>
+      </c>
+      <c r="D2" s="11" t="inlineStr">
+        <is>
+          <t>晚期 1L + III 期辅助 + IIB/IIC 辅助</t>
+        </is>
+      </c>
+      <c r="E2" s="45" t="n">
+        <v>112000</v>
+      </c>
+      <c r="F2" s="45" t="n">
+        <v>1500000</v>
+      </c>
+      <c r="G2" s="11" t="inlineStr">
+        <is>
+          <t>黑色素瘤 112,000 → 晚期 + 高危可辅助人群约 25% = 28,000 → 接受免疫治疗 30% = 8,400</t>
+        </is>
+      </c>
+      <c r="H2" s="46" t="n">
+        <v>28000</v>
+      </c>
+      <c r="I2" s="47" t="n">
+        <v>8400</v>
+      </c>
+      <c r="J2" s="48" t="n">
+        <v>1</v>
+      </c>
+      <c r="K2" s="49" t="n">
+        <v>213299.0476190476</v>
+      </c>
+      <c r="L2" s="49" t="n">
+        <v>198880.7277628032</v>
+      </c>
+      <c r="M2" s="50" t="n">
+        <v>5972.4</v>
+      </c>
+      <c r="N2" s="51" t="n">
+        <v>1670.6</v>
+      </c>
+      <c r="O2" s="52" t="n">
+        <v>0.2797209785737129</v>
+      </c>
+      <c r="P2" s="11" t="inlineStr">
+        <is>
+          <t>KEYNOTE-001/006/054/716 四项批准；AK112 无任何黑色素瘤研究</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="43" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="11" t="inlineStr">
+        <is>
+          <t>K药 独占（AK112 空白）</t>
+        </is>
+      </c>
+      <c r="C3" s="44" t="inlineStr">
+        <is>
+          <t>经典霍奇金淋巴瘤</t>
+        </is>
+      </c>
+      <c r="D3" s="11" t="inlineStr">
+        <is>
+          <t>复发/难治</t>
+        </is>
+      </c>
+      <c r="E3" s="45" t="n">
+        <v>8920</v>
+      </c>
+      <c r="F3" s="45" t="n">
+        <v>230000</v>
+      </c>
+      <c r="G3" s="11" t="inlineStr">
+        <is>
+          <t>cHL 8,920 → 复发/难治约 20% = 1,784 → 接受 PD-1 治疗 60% = 1,070</t>
+        </is>
+      </c>
+      <c r="H3" s="46" t="n">
+        <v>1784</v>
+      </c>
+      <c r="I3" s="47" t="n">
+        <v>1070</v>
+      </c>
+      <c r="J3" s="48" t="n">
+        <v>1</v>
+      </c>
+      <c r="K3" s="49" t="n">
+        <v>213299.0476190476</v>
+      </c>
+      <c r="L3" s="49" t="n">
+        <v>198880.7277628032</v>
+      </c>
+      <c r="M3" s="50" t="n">
+        <v>380.5</v>
+      </c>
+      <c r="N3" s="51" t="n">
+        <v>212.8</v>
+      </c>
+      <c r="O3" s="52" t="n">
+        <v>0.5592328981200911</v>
+      </c>
+      <c r="P3" s="11" t="inlineStr">
+        <is>
+          <t>ORR 65–73%、PFS HR 0.65；AK112 无任何血液瘤研究</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="43" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="11" t="inlineStr">
+        <is>
+          <t>K药 独占（AK112 空白）</t>
+        </is>
+      </c>
+      <c r="C4" s="44" t="inlineStr">
+        <is>
+          <t>泛癌 MSI-H / dMMR</t>
+        </is>
+      </c>
+      <c r="D4" s="11" t="inlineStr">
+        <is>
+          <t>既往治疗失败（不依器官）</t>
+        </is>
+      </c>
+      <c r="E4" s="45" t="n">
+        <v>24000</v>
+      </c>
+      <c r="F4" s="45" t="n"/>
+      <c r="G4" s="11" t="inlineStr">
+        <is>
+          <t>美国晚期实体瘤年治疗池约 600,000 → MSI-H/dMMR 约 4% = 24,000 → 接受治疗 35% = 8,400</t>
+        </is>
+      </c>
+      <c r="H4" s="46" t="n">
+        <v>24000</v>
+      </c>
+      <c r="I4" s="47" t="n">
+        <v>8400</v>
+      </c>
+      <c r="J4" s="48" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="K4" s="49" t="n">
+        <v>213299.0476190476</v>
+      </c>
+      <c r="L4" s="49" t="n">
+        <v>198880.7277628032</v>
+      </c>
+      <c r="M4" s="50" t="n">
+        <v>7678.8</v>
+      </c>
+      <c r="N4" s="51" t="n">
+        <v>2505.9</v>
+      </c>
+      <c r="O4" s="52" t="n">
+        <v>0.3263411416693316</v>
+      </c>
+      <c r="P4" s="11" t="inlineStr">
+        <is>
+          <t>史上首个不依器官批准，ORR 34–71%，DOR 极长（治疗时长 1.5 年）；AK112 从未做分子富集队列</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="43" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t>K药 独占（AK112 空白）</t>
+        </is>
+      </c>
+      <c r="C5" s="44" t="inlineStr">
+        <is>
+          <t>泛癌 TMB-H（≥10 mut/Mb）</t>
+        </is>
+      </c>
+      <c r="D5" s="11" t="inlineStr">
+        <is>
+          <t>既往治疗失败</t>
+        </is>
+      </c>
+      <c r="E5" s="45" t="n">
+        <v>15000</v>
+      </c>
+      <c r="F5" s="45" t="n"/>
+      <c r="G5" s="11" t="inlineStr">
+        <is>
+          <t>晚期实体瘤中 TMB-H（排除 dMMR）约 2.5% = 15,000 → 接受治疗 15% = 2,250</t>
+        </is>
+      </c>
+      <c r="H5" s="46" t="n">
+        <v>15000</v>
+      </c>
+      <c r="I5" s="47" t="n">
+        <v>2250</v>
+      </c>
+      <c r="J5" s="48" t="n">
+        <v>1</v>
+      </c>
+      <c r="K5" s="49" t="n">
+        <v>213299.0476190476</v>
+      </c>
+      <c r="L5" s="49" t="n">
+        <v>198880.7277628032</v>
+      </c>
+      <c r="M5" s="50" t="n">
+        <v>3199.5</v>
+      </c>
+      <c r="N5" s="51" t="n">
+        <v>447.5</v>
+      </c>
+      <c r="O5" s="52" t="n">
+        <v>0.1398604892868564</v>
+      </c>
+      <c r="P5" s="11" t="inlineStr">
+        <is>
+          <t>ORR 29%，学界对通用阈值争议大；AK112 无 TMB 分层开发</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="43" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="11" t="inlineStr">
+        <is>
+          <t>K药 独占（AK112 空白）</t>
+        </is>
+      </c>
+      <c r="C6" s="44" t="inlineStr">
+        <is>
+          <t>Merkel 细胞癌</t>
+        </is>
+      </c>
+      <c r="D6" s="11" t="inlineStr">
+        <is>
+          <t>复发局晚/转移 一线</t>
+        </is>
+      </c>
+      <c r="E6" s="45" t="n">
+        <v>3000</v>
+      </c>
+      <c r="F6" s="45" t="n">
+        <v>4500</v>
+      </c>
+      <c r="G6" s="11" t="inlineStr">
+        <is>
+          <t>MCC 约 3,000 → 复发局晚/转移 25% = 750 → 接受治疗 50% = 375</t>
+        </is>
+      </c>
+      <c r="H6" s="46" t="n">
+        <v>750</v>
+      </c>
+      <c r="I6" s="47" t="n">
+        <v>375</v>
+      </c>
+      <c r="J6" s="48" t="n">
+        <v>1</v>
+      </c>
+      <c r="K6" s="49" t="n">
+        <v>213299.0476190476</v>
+      </c>
+      <c r="L6" s="49" t="n">
+        <v>198880.7277628032</v>
+      </c>
+      <c r="M6" s="50" t="n">
+        <v>160</v>
+      </c>
+      <c r="N6" s="51" t="n">
+        <v>74.59999999999999</v>
+      </c>
+      <c r="O6" s="52" t="n">
+        <v>0.4662016309561881</v>
+      </c>
+      <c r="P6" s="11" t="inlineStr">
+        <is>
+          <t>ORR 56%、3 年 OS 59%；AK112 无</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="43" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>K药 独占（AK112 空白）</t>
+        </is>
+      </c>
+      <c r="C7" s="44" t="inlineStr">
+        <is>
+          <t>皮肤鳞癌（cSCC）</t>
+        </is>
+      </c>
+      <c r="D7" s="11" t="inlineStr">
+        <is>
+          <t>复发/转移 或 局晚不可手术</t>
+        </is>
+      </c>
+      <c r="E7" s="45" t="n">
+        <v>15000</v>
+      </c>
+      <c r="F7" s="45" t="n"/>
+      <c r="G7" s="11" t="inlineStr">
+        <is>
+          <t>cSCC 年发病超百万，但晚期/不可切除仅约 15,000 → 接受治疗 30% = 4,500</t>
+        </is>
+      </c>
+      <c r="H7" s="46" t="n">
+        <v>15000</v>
+      </c>
+      <c r="I7" s="47" t="n">
+        <v>4500</v>
+      </c>
+      <c r="J7" s="48" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="K7" s="49" t="n">
+        <v>213299.0476190476</v>
+      </c>
+      <c r="L7" s="49" t="n">
+        <v>198880.7277628032</v>
+      </c>
+      <c r="M7" s="50" t="n">
+        <v>2559.6</v>
+      </c>
+      <c r="N7" s="51" t="n">
+        <v>716</v>
+      </c>
+      <c r="O7" s="52" t="n">
+        <v>0.2797209785737129</v>
+      </c>
+      <c r="P7" s="11" t="inlineStr">
+        <is>
+          <t>ORR 35–50% 已获批（但辅助 KEYNOTE-630 失败，OS HR 1.47）；AK112 仅 1 项 IIT 无读出</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="43" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>K药 独占（AK112 空白）</t>
+        </is>
+      </c>
+      <c r="C8" s="44" t="inlineStr">
+        <is>
+          <t>尿路上皮癌 / 膀胱癌</t>
+        </is>
+      </c>
+      <c r="D8" s="11" t="inlineStr">
+        <is>
+          <t>晚期 1L(+EV) / 2L / NMIBC CIS / MIBC 围手术期</t>
+        </is>
+      </c>
+      <c r="E8" s="45" t="n">
+        <v>84530</v>
+      </c>
+      <c r="F8" s="45" t="n">
+        <v>730000</v>
+      </c>
+      <c r="G8" s="11" t="inlineStr">
+        <is>
+          <t>膀胱 84,530 → 晚期 + MIBC 围手术期 + NMIBC CIS 合计可及约 22,000 → 接受治疗 40% = 8,800</t>
+        </is>
+      </c>
+      <c r="H8" s="46" t="n">
+        <v>22000</v>
+      </c>
+      <c r="I8" s="47" t="n">
+        <v>8800</v>
+      </c>
+      <c r="J8" s="48" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="K8" s="49" t="n">
+        <v>213299.0476190476</v>
+      </c>
+      <c r="L8" s="49" t="n">
+        <v>198880.7277628032</v>
+      </c>
+      <c r="M8" s="50" t="n">
+        <v>4223.3</v>
+      </c>
+      <c r="N8" s="51" t="n">
+        <v>1575.1</v>
+      </c>
+      <c r="O8" s="52" t="n">
+        <v>0.3729613047649505</v>
+      </c>
+      <c r="P8" s="11" t="inlineStr">
+        <is>
+          <t>四个适应症：EV-302 OS HR 0.47（全项目最强）、KEYNOTE-045、-057、-905；AK112 仅 1 项 IIT</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="43" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="11" t="inlineStr">
+        <is>
+          <t>K药 独占（AK112 空白）</t>
+        </is>
+      </c>
+      <c r="C9" s="44" t="inlineStr">
+        <is>
+          <t>肾细胞癌（RCC）</t>
+        </is>
+      </c>
+      <c r="D9" s="11" t="inlineStr">
+        <is>
+          <t>晚期 1L(+阿昔替尼) + 术后辅助</t>
+        </is>
+      </c>
+      <c r="E9" s="45" t="n">
+        <v>80450</v>
+      </c>
+      <c r="F9" s="45" t="n">
+        <v>600000</v>
+      </c>
+      <c r="G9" s="11" t="inlineStr">
+        <is>
+          <t>肾癌 80,450 → 晚期 + 中高危可辅助约 24,000 → 接受治疗 35% = 8,400</t>
+        </is>
+      </c>
+      <c r="H9" s="46" t="n">
+        <v>24000</v>
+      </c>
+      <c r="I9" s="47" t="n">
+        <v>8400</v>
+      </c>
+      <c r="J9" s="48" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="K9" s="49" t="n">
+        <v>213299.0476190476</v>
+      </c>
+      <c r="L9" s="49" t="n">
+        <v>198880.7277628032</v>
+      </c>
+      <c r="M9" s="50" t="n">
+        <v>6143</v>
+      </c>
+      <c r="N9" s="51" t="n">
+        <v>2004.7</v>
+      </c>
+      <c r="O9" s="52" t="n">
+        <v>0.3263411416693316</v>
+      </c>
+      <c r="P9" s="11" t="inlineStr">
+        <is>
+          <t>KEYNOTE-426 OS HR 0.68、KEYNOTE-564 辅助 OS HR 0.62（首个辅助免疫 OS 阳性）；AK112 仅 2 项 IIT</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="43" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="11" t="inlineStr">
+        <is>
+          <t>K药 独占（AK112 空白）</t>
+        </is>
+      </c>
+      <c r="C10" s="44" t="inlineStr">
+        <is>
+          <t>三阴性乳腺癌（早期）</t>
+        </is>
+      </c>
+      <c r="D10" s="11" t="inlineStr">
+        <is>
+          <t>II–III 期 新辅助 + 辅助</t>
+        </is>
+      </c>
+      <c r="E10" s="45" t="n">
+        <v>38950</v>
+      </c>
+      <c r="F10" s="45" t="n"/>
+      <c r="G10" s="11" t="inlineStr">
+        <is>
+          <t>TNBC 38,950 → II–III 期可手术 55% = 21,423 → 接受围手术期免疫 55% = 11,782</t>
+        </is>
+      </c>
+      <c r="H10" s="46" t="n">
+        <v>21423</v>
+      </c>
+      <c r="I10" s="47" t="n">
+        <v>11782</v>
+      </c>
+      <c r="J10" s="48" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="K10" s="49" t="n">
+        <v>213299.0476190476</v>
+      </c>
+      <c r="L10" s="49" t="n">
+        <v>198880.7277628032</v>
+      </c>
+      <c r="M10" s="50" t="n">
+        <v>4112.6</v>
+      </c>
+      <c r="N10" s="51" t="n">
+        <v>2108.9</v>
+      </c>
+      <c r="O10" s="52" t="n">
+        <v>0.5127935037973961</v>
+      </c>
+      <c r="P10" s="11" t="inlineStr">
+        <is>
+          <t>KEYNOTE-522 pCR 64.8%、EFS HR 0.63、OS HR 0.66（唯一 OS 阳性的早期 TNBC 免疫方案）；AK112 仅 IIT</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="43" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="11" t="inlineStr">
+        <is>
+          <t>K药 独占（AK112 空白）</t>
+        </is>
+      </c>
+      <c r="C11" s="44" t="inlineStr">
+        <is>
+          <t>食管癌 / GEJ</t>
+        </is>
+      </c>
+      <c r="D11" s="11" t="inlineStr">
+        <is>
+          <t>局晚/转移 一线 +化疗</t>
+        </is>
+      </c>
+      <c r="E11" s="45" t="n">
+        <v>22530</v>
+      </c>
+      <c r="F11" s="45" t="n">
+        <v>50000</v>
+      </c>
+      <c r="G11" s="11" t="inlineStr">
+        <is>
+          <t>食管 22,530 → 晚期/转移 65% = 14,645 → 接受一线治疗 40% = 5,858</t>
+        </is>
+      </c>
+      <c r="H11" s="46" t="n">
+        <v>14645</v>
+      </c>
+      <c r="I11" s="47" t="n">
+        <v>5858</v>
+      </c>
+      <c r="J11" s="48" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="K11" s="49" t="n">
+        <v>213299.0476190476</v>
+      </c>
+      <c r="L11" s="49" t="n">
+        <v>198880.7277628032</v>
+      </c>
+      <c r="M11" s="50" t="n">
+        <v>1874.3</v>
+      </c>
+      <c r="N11" s="51" t="n">
+        <v>699</v>
+      </c>
+      <c r="O11" s="52" t="n">
+        <v>0.3729613047649504</v>
+      </c>
+      <c r="P11" s="11" t="inlineStr">
+        <is>
+          <t>KEYNOTE-590 OS HR 0.73；AK112 仅 5 项 IIT 无读出，且 LEAP-014 同类思路在 K药 侧亦失败</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="43" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="11" t="inlineStr">
+        <is>
+          <t>K药 独占（AK112 空白）</t>
+        </is>
+      </c>
+      <c r="C12" s="44" t="inlineStr">
+        <is>
+          <t>宫颈癌（一线 + 局部晚期）</t>
+        </is>
+      </c>
+      <c r="D12" s="11" t="inlineStr">
+        <is>
+          <t>1L 复发/转移 +化疗±bev；局晚 同步放化疗</t>
+        </is>
+      </c>
+      <c r="E12" s="45" t="n">
+        <v>13490</v>
+      </c>
+      <c r="F12" s="45" t="n">
+        <v>290000</v>
+      </c>
+      <c r="G12" s="11" t="inlineStr">
+        <is>
+          <t>宫颈 13,490 → 一线复发转移 + 局晚可及约 55% = 7,420 → 接受治疗 45% = 3,339</t>
+        </is>
+      </c>
+      <c r="H12" s="46" t="n">
+        <v>7420</v>
+      </c>
+      <c r="I12" s="47" t="n">
+        <v>3339</v>
+      </c>
+      <c r="J12" s="48" t="n">
+        <v>1</v>
+      </c>
+      <c r="K12" s="49" t="n">
+        <v>213299.0476190476</v>
+      </c>
+      <c r="L12" s="49" t="n">
+        <v>198880.7277628032</v>
+      </c>
+      <c r="M12" s="50" t="n">
+        <v>1582.7</v>
+      </c>
+      <c r="N12" s="51" t="n">
+        <v>664.1</v>
+      </c>
+      <c r="O12" s="52" t="n">
+        <v>0.4195814678605693</v>
+      </c>
+      <c r="P12" s="11" t="inlineStr">
+        <is>
+          <t>KEYNOTE-826 OS HR 0.60、KEYNOTE-A18 OS HR 0.67；AK112 仅 IIT 且场景已挪到早期新辅助</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="43" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="11" t="inlineStr">
+        <is>
+          <t>K药 独占（AK112 空白）</t>
+        </is>
+      </c>
+      <c r="C13" s="44" t="inlineStr">
+        <is>
+          <t>NSCLC 术后辅助</t>
+        </is>
+      </c>
+      <c r="D13" s="11" t="inlineStr">
+        <is>
+          <t>IB–IIIA 期 完全切除后</t>
+        </is>
+      </c>
+      <c r="E13" s="45" t="n">
+        <v>195000</v>
+      </c>
+      <c r="F13" s="45" t="n">
+        <v>625000</v>
+      </c>
+      <c r="G13" s="11" t="inlineStr">
+        <is>
+          <t>NSCLC 195,000 → I–IIIA 可切除并完成手术约 22% = 42,900 → 接受辅助免疫 20% = 8,580</t>
+        </is>
+      </c>
+      <c r="H13" s="46" t="n">
+        <v>42900</v>
+      </c>
+      <c r="I13" s="47" t="n">
+        <v>8580</v>
+      </c>
+      <c r="J13" s="48" t="n">
+        <v>1</v>
+      </c>
+      <c r="K13" s="49" t="n">
+        <v>213299.0476190476</v>
+      </c>
+      <c r="L13" s="49" t="n">
+        <v>198880.7277628032</v>
+      </c>
+      <c r="M13" s="50" t="n">
+        <v>9150.5</v>
+      </c>
+      <c r="N13" s="51" t="n">
+        <v>1706.4</v>
+      </c>
+      <c r="O13" s="52" t="n">
+        <v>0.1864806523824752</v>
+      </c>
+      <c r="P13" s="11" t="inlineStr">
+        <is>
+          <t>KEYNOTE-091 全体 DFS HR 0.76（但 PD-L1≥50% 亚组未达）；AK112 无术后单纯辅助研究</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="43" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="11" t="inlineStr">
+        <is>
+          <t>K药 独占（AK112 空白）</t>
+        </is>
+      </c>
+      <c r="C14" s="44" t="inlineStr">
+        <is>
+          <t>胃癌 HER2 阳性</t>
+        </is>
+      </c>
+      <c r="D14" s="11" t="inlineStr">
+        <is>
+          <t>一线 +曲妥珠单抗+化疗</t>
+        </is>
+      </c>
+      <c r="E14" s="45" t="n">
+        <v>38270</v>
+      </c>
+      <c r="F14" s="45" t="n">
+        <v>130000</v>
+      </c>
+      <c r="G14" s="11" t="inlineStr">
+        <is>
+          <t>胃/GEJ 38,270 → 晚期 60% × HER2 阳性 20% = 4,592 → 接受治疗 40% = 1,837</t>
+        </is>
+      </c>
+      <c r="H14" s="46" t="n">
+        <v>4592</v>
+      </c>
+      <c r="I14" s="47" t="n">
+        <v>1837</v>
+      </c>
+      <c r="J14" s="48" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="K14" s="49" t="n">
+        <v>213299.0476190476</v>
+      </c>
+      <c r="L14" s="49" t="n">
+        <v>198880.7277628032</v>
+      </c>
+      <c r="M14" s="50" t="n">
+        <v>783.6</v>
+      </c>
+      <c r="N14" s="51" t="n">
+        <v>292.3</v>
+      </c>
+      <c r="O14" s="52" t="n">
+        <v>0.3730019146631174</v>
+      </c>
+      <c r="P14" s="11" t="inlineStr">
+        <is>
+          <t>KEYNOTE-811 ORR 74% vs 52%、PFS HR 0.72；AK112 无 HER2 分层开发</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="55" t="n"/>
+      <c r="B15" s="56" t="inlineStr">
+        <is>
+          <t>合计</t>
+        </is>
+      </c>
+      <c r="C15" s="57" t="n"/>
+      <c r="D15" s="56" t="n"/>
+      <c r="E15" s="58" t="n"/>
+      <c r="F15" s="58" t="n"/>
+      <c r="G15" s="56" t="inlineStr">
+        <is>
+          <t>注：合计仅供量级校准；同一瘤种不同线数存在患者池重叠，不可简单相加</t>
+        </is>
+      </c>
+      <c r="H15" s="58" t="n"/>
+      <c r="I15" s="58" t="n"/>
+      <c r="J15" s="59" t="n"/>
+      <c r="K15" s="60" t="n"/>
+      <c r="L15" s="60" t="n"/>
+      <c r="M15" s="61" t="n">
+        <v>47820.6</v>
+      </c>
+      <c r="N15" s="61" t="n">
+        <v>14677.8</v>
+      </c>
+      <c r="O15" s="62" t="n">
+        <v>0.3069351231551667</v>
+      </c>
+      <c r="P15" s="56" t="n"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:P14"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B39"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="126" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>美国价格与测算口径（2026-03）</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr"/>
+      <c r="B2" s="4" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>K药 标价（WAC / list）</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>$12,272 / 200mg（Q3W）；$24,544 / 400mg（Q6W）—— 两者每周单价完全相同。来源：Merck 官方患者网站，标注 current as of March 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>K药 标价年化</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>$213,299 / 患者·年（17.38 个 Q3W 周期）</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>K药 实付（Medicare Part B 净 ASP）</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>J9271 Q3-2026 支付上限 $60.645/mg = ASP+6% → 剥离加成后净 ASP = $11,442 / 200mg</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>K药 实付年化</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>$198,881 / 患者·年（约为标价的 93%）</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>为什么美国标价与实付只差约 7%</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>K药 是院内输注的 Part B buy-and-bill 药物，不走 PBM 零售回扣体系，返利空间远小于 Part D 口服药。这与中国「标价 vs 赠药后实付」可差 2–5 倍完全不同</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>商业保险实际议价区间</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>各州各支付方对 200mg 的议价区间为 $12,000 至 $30,000+（同地区不同机构可差 5–10 倍），主要由计费类别、服务场所与议价能力决定，非临床因素。本表统一用 ASP 净价，属保守口径</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Medicare 实际到手</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>ASP+6% 再扣 2% sequestration → 实际约 ASP+4.3% ≈ $11,935 / 200mg</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr"/>
+      <c r="B10" s="4" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>AK112 美国价格</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>**尚未上市，Summit 从未披露定价。本表统一按与 K药 净价平价假设，纯属占位。**</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>AK112 定价的成本约束</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>依沃西 20mg/kg Q3W，70kg 患者单次 1,400mg，是 K药 200mg 的约 7 倍蛋白量。COGS 显著更高，构成定价下限约束——难以低价竞争</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>AK112 定价三情景（供自行替换）</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>平价 $198,881；OS 优效标签溢价 15% = $228,713；仅 PFS 标签需折价 10% = $178,993</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr"/>
+      <c r="B14" s="4" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>市场空间算法</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>空间 = 可及患者数 × 平均治疗时长（年）× 年化费用</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>为什么必须乘治疗时长</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>绝大多数晚期适应症的患者治疗不满一年（如 ES-SCLC 仅 0.45 年、间皮瘤 0.35 年）。直接用「患者数 × 年费用」会系统性高估 30–60%。本表已单列治疗时长，可自行调整</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>天花板情景</t>
+        </is>
+      </c>
+      <c r="B17" s="4">
+        <f> 全部符合分期/biomarker 条件的患者（不打治疗渗透率、不打竞争份额）× 治疗时长 × **标价**。用途：判断适应症的物理上限</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>现实情景</t>
+        </is>
+      </c>
+      <c r="B18" s="4">
+        <f> 天花板 → 再乘治疗渗透率 → 再乘竞争份额假设 × 治疗时长 × **实付净价**。用途：贴近可实现峰值销售</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>份额假设已逐行标注</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>见每行最后一列。份额是本表最主观的变量，请务必自行替换后再使用</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr"/>
+      <c r="B20" s="4" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="1" t="inlineStr">
+        <is>
+          <t>数据来源</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>发病数</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>ACS《Cancer Statistics, 2026》Table 1（CA: A Cancer Journal for Clinicians，2026-01-13 发布）。全美 2026 年预计新发 2,114,850 例。所有「瘤种新发」列均为该表实测值，未做调整</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>现存患者数</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>SEER 全病程 prevalence 近似值（非 5 年 prevalence），仅作背景参考。**晚期免疫治疗的市场空间由年治疗池驱动，存量列不参与任何计算**</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>分期 / biomarker / 渗透率占比</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>均为文献与流行病学惯用值的推算，非官方统计。每行「目标人群推算链」列已把每一步乘数写明，可逐步复核与替换</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>价格</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>Merck 官方 WAC 页（2026-03）、CMS Medicare Part B ASP 定价文件（J9271, Q3-2026）</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr"/>
+      <c r="B26" s="4" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="1" t="inlineStr">
+        <is>
+          <t>校准检验</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>Keytruda 实际销售额</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>2025 年全球 $316.8 亿（含 Keytruda Qlex），美国约占 55% ≈ $174 亿；2025 Q4 单季 $83.7 亿</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>反推患者年</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>$174 亿 ÷ $198,881 ≈ 87,500 患者·年。本表「K药 独占领域 + 配对适应症中 K药 已获批部分」的现实情景合计应落在同一量级，否则份额假设需下调</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr"/>
+      <c r="B30" s="4" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>免责</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>本表为公开信息整理与情景推算，所有占比与份额均为假设，不构成任何医疗建议或投资建议。发病数与价格可核验，患者分层与份额不可核验</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="63" t="inlineStr">
+        <is>
+          <t>【实测校准结果 —— 请务必先读】</t>
+        </is>
+      </c>
+      <c r="B32" s="64" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="38" t="inlineStr">
+        <is>
+          <t>本表现实情景合计</t>
+        </is>
+      </c>
+      <c r="B33" s="65" t="inlineStr">
+        <is>
+          <t>配对适应症 $110.7 亿 + K药独占领域 $146.8 亿 = **$257.4 亿/年**</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="38" t="inlineStr">
+        <is>
+          <t>Keytruda 美国实际销售额</t>
+        </is>
+      </c>
+      <c r="B34" s="65" t="inlineStr">
+        <is>
+          <t>约 **$174 亿/年**（2025 年全球 $316.8 亿 × 美国占比约 55%）</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="38" t="inlineStr">
+        <is>
+          <t>结论：本表整体偏高</t>
+        </is>
+      </c>
+      <c r="B35" s="65" t="inlineStr">
+        <is>
+          <t>剔除纯 AK112 场景（IO 耐药 NSCLC、胰腺癌、MSS CRC 一线、EGFR 二线、CPS&lt;10 TNBC，合计约 $36 亿）后，可归属 K药 的现实情景约 $222 亿，仍比实际高约 27%。</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="38" t="inlineStr">
+        <is>
+          <t>偏高的三个来源</t>
+        </is>
+      </c>
+      <c r="B36" s="65" t="inlineStr">
+        <is>
+          <t>①竞争份额假设（15%–45%）整体偏乐观；②「接受治疗渗透率」在真实世界更低（体能状态、合并症、患者拒治、可及性）；③同一瘤种不同线数的患者池存在重叠，横向相加会重复计数</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="38" t="inlineStr">
+        <is>
+          <t>**建议用法**</t>
+        </is>
+      </c>
+      <c r="B37" s="65" t="inlineStr">
+        <is>
+          <t>把「现实情景空间」整体乘 0.7–0.75 作为校准系数后再使用；或直接把各行的竞争份额假设下调三分之一。天花板列不受此影响（它本就是物理上限，不含份额假设）</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="38" t="inlineStr">
+        <is>
+          <t>为什么保留未校准的原值</t>
+        </is>
+      </c>
+      <c r="B38" s="65" t="inlineStr">
+        <is>
+          <t>校准系数应由使用者按自己的份额判断施加，而非我在数据里预先抹平。逐行份额假设已写在最后一列，便于替换</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="38" t="inlineStr"/>
+      <c r="B39" s="65" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3155,7 +6109,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="30" t="n">
+      <c r="A2" s="43" t="n">
         <v>1</v>
       </c>
       <c r="B2" s="10" t="inlineStr">
@@ -3168,7 +6122,7 @@
           <t>★★★★★ 瘤种/线数/期别/联合方案/对照设计 全部对等</t>
         </is>
       </c>
-      <c r="D2" s="32" t="inlineStr">
+      <c r="D2" s="44" t="inlineStr">
         <is>
           <t>NSCLC（非鳞，EGFR 突变）</t>
         </is>
@@ -3230,7 +6184,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="30" t="n">
+      <c r="A3" s="43" t="n">
         <v>2</v>
       </c>
       <c r="B3" s="10" t="inlineStr">
@@ -3243,7 +6197,7 @@
           <t>★★★★☆ 同上，但仅 PFS 达标（全球人群）</t>
         </is>
       </c>
-      <c r="D3" s="32" t="inlineStr">
+      <c r="D3" s="44" t="inlineStr">
         <is>
           <t>NSCLC（非鳞，EGFR 突变）</t>
         </is>
@@ -3305,7 +6259,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="30" t="n">
+      <c r="A4" s="43" t="n">
         <v>3</v>
       </c>
       <c r="B4" s="35" t="inlineStr">
@@ -3318,7 +6272,7 @@
           <t>★★★☆☆ 同瘤种/同线数/同期别/同类方案，但样本小、差距不显著</t>
         </is>
       </c>
-      <c r="D4" s="32" t="inlineStr">
+      <c r="D4" s="44" t="inlineStr">
         <is>
           <t>结直肠癌（MSS/pMMR）</t>
         </is>
@@ -3380,7 +6334,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="30" t="n">
+      <c r="A5" s="43" t="n">
         <v>4</v>
       </c>
       <c r="B5" s="35" t="inlineStr">
@@ -3393,7 +6347,7 @@
           <t>★★★☆☆ 同瘤种/同线数/同期别，但方案不对等（联合 vs 单药）</t>
         </is>
       </c>
-      <c r="D5" s="32" t="inlineStr">
+      <c r="D5" s="44" t="inlineStr">
         <is>
           <t>三阴性乳腺癌（TNBC）</t>
         </is>
@@ -3455,7 +6409,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="30" t="n">
+      <c r="A6" s="43" t="n">
         <v>5</v>
       </c>
       <c r="B6" s="35" t="inlineStr">
@@ -3468,7 +6422,7 @@
           <t>★★☆☆☆ 同瘤种/同线数/同方案（单药），但样本量差 20 倍</t>
         </is>
       </c>
-      <c r="D6" s="32" t="inlineStr">
+      <c r="D6" s="44" t="inlineStr">
         <is>
           <t>卵巢癌 / 输卵管 / 原发腹膜癌</t>
         </is>
@@ -3530,7 +6484,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="30" t="n">
+      <c r="A7" s="43" t="n">
         <v>6</v>
       </c>
       <c r="B7" s="19" t="inlineStr">
@@ -3543,7 +6497,7 @@
           <t>不符合筛选条件，但价值最高：K药 被头对头击败</t>
         </is>
       </c>
-      <c r="D7" s="32" t="inlineStr">
+      <c r="D7" s="44" t="inlineStr">
         <is>
           <t>NSCLC</t>
         </is>
@@ -3605,7 +6559,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="30" t="n">
+      <c r="A8" s="43" t="n">
         <v>7</v>
       </c>
       <c r="B8" s="19" t="inlineStr">
@@ -3618,7 +6572,7 @@
           <t>两者均成功，未头对头</t>
         </is>
       </c>
-      <c r="D8" s="32" t="inlineStr">
+      <c r="D8" s="44" t="inlineStr">
         <is>
           <t>NSCLC（鳞）</t>
         </is>
@@ -3680,7 +6634,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="30" t="n">
+      <c r="A9" s="43" t="n">
         <v>8</v>
       </c>
       <c r="B9" s="19" t="inlineStr">
@@ -3693,7 +6647,7 @@
           <t>两者均成功，对照强度差一个量级</t>
         </is>
       </c>
-      <c r="D9" s="32" t="inlineStr">
+      <c r="D9" s="44" t="inlineStr">
         <is>
           <t>胆道癌（BTC）</t>
         </is>
@@ -3755,7 +6709,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="30" t="n">
+      <c r="A10" s="43" t="n">
         <v>9</v>
       </c>
       <c r="B10" s="19" t="inlineStr">
@@ -3768,7 +6722,7 @@
           <t>K药 已 III 期成功，AK112 仅 II 期单臂</t>
         </is>
       </c>
-      <c r="D10" s="32" t="inlineStr">
+      <c r="D10" s="44" t="inlineStr">
         <is>
           <t>NSCLC</t>
         </is>
@@ -3830,7 +6784,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="30" t="n">
+      <c r="A11" s="43" t="n">
         <v>10</v>
       </c>
       <c r="B11" s="19" t="inlineStr">
@@ -3843,7 +6797,7 @@
           <t>K药 已 III 期成功，AK112 仅单中心 IIT</t>
         </is>
       </c>
-      <c r="D11" s="32" t="inlineStr">
+      <c r="D11" s="44" t="inlineStr">
         <is>
           <t>头颈鳞癌（HNSCC）</t>
         </is>
@@ -3905,7 +6859,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="30" t="n">
+      <c r="A12" s="43" t="n">
         <v>11</v>
       </c>
       <c r="B12" s="19" t="inlineStr">
@@ -3918,7 +6872,7 @@
           <t>K药 已 III 期成功，同期别 ORR 差距有限</t>
         </is>
       </c>
-      <c r="D12" s="32" t="inlineStr">
+      <c r="D12" s="44" t="inlineStr">
         <is>
           <t>胃 / 胃食管结合部腺癌</t>
         </is>
@@ -3980,7 +6934,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="30" t="n">
+      <c r="A13" s="43" t="n">
         <v>12</v>
       </c>
       <c r="B13" s="36" t="inlineStr">
@@ -3993,7 +6947,7 @@
           <t>K药 机制上不适用，不应计入战绩对比</t>
         </is>
       </c>
-      <c r="D13" s="32" t="inlineStr">
+      <c r="D13" s="44" t="inlineStr">
         <is>
           <t>NSCLC</t>
         </is>
@@ -4055,7 +7009,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="30" t="n">
+      <c r="A14" s="43" t="n">
         <v>13</v>
       </c>
       <c r="B14" s="36" t="inlineStr">
@@ -4068,7 +7022,7 @@
           <t>K药 明确失败，但 AK112 数据未公开，无法比较</t>
         </is>
       </c>
-      <c r="D14" s="32" t="inlineStr">
+      <c r="D14" s="44" t="inlineStr">
         <is>
           <t>胰腺癌（PDAC）</t>
         </is>
@@ -4130,7 +7084,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="30" t="n">
+      <c r="A15" s="43" t="n">
         <v>14</v>
       </c>
       <c r="B15" s="36" t="inlineStr">
@@ -4143,7 +7097,7 @@
           <t>期别相差三级，且 AK112 自己也未验证</t>
         </is>
       </c>
-      <c r="D15" s="32" t="inlineStr">
+      <c r="D15" s="44" t="inlineStr">
         <is>
           <t>小细胞肺癌（SCLC）</t>
         </is>
@@ -4205,7 +7159,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="30" t="n">
+      <c r="A16" s="43" t="n">
         <v>15</v>
       </c>
       <c r="B16" s="36" t="inlineStr">
@@ -4218,7 +7172,7 @@
           <t>方案不对等（联合 vs 单药），且 K药 最终在 III 期成功</t>
         </is>
       </c>
-      <c r="D16" s="32" t="inlineStr">
+      <c r="D16" s="44" t="inlineStr">
         <is>
           <t>胆道癌（BTC）</t>
         </is>
@@ -4389,7 +7343,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="30" t="n">
+      <c r="A2" s="43" t="n">
         <v>1</v>
       </c>
       <c r="B2" s="10" t="inlineStr">
@@ -4402,7 +7356,7 @@
           <t>★★★★★ 瘤种/线数/期别/联合方案/对照设计 全部对等</t>
         </is>
       </c>
-      <c r="D2" s="32" t="inlineStr">
+      <c r="D2" s="44" t="inlineStr">
         <is>
           <t>NSCLC（非鳞，EGFR 突变）</t>
         </is>
@@ -4464,7 +7418,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="30" t="n">
+      <c r="A3" s="43" t="n">
         <v>2</v>
       </c>
       <c r="B3" s="10" t="inlineStr">
@@ -4477,7 +7431,7 @@
           <t>★★★★☆ 同上，但仅 PFS 达标（全球人群）</t>
         </is>
       </c>
-      <c r="D3" s="32" t="inlineStr">
+      <c r="D3" s="44" t="inlineStr">
         <is>
           <t>NSCLC（非鳞，EGFR 突变）</t>
         </is>
@@ -4648,7 +7602,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="30" t="n">
+      <c r="A2" s="43" t="n">
         <v>1</v>
       </c>
       <c r="B2" s="35" t="inlineStr">
@@ -4661,7 +7615,7 @@
           <t>★★★☆☆ 同瘤种/同线数/同期别/同类方案，但样本小、差距不显著</t>
         </is>
       </c>
-      <c r="D2" s="32" t="inlineStr">
+      <c r="D2" s="44" t="inlineStr">
         <is>
           <t>结直肠癌（MSS/pMMR）</t>
         </is>
@@ -4723,7 +7677,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="30" t="n">
+      <c r="A3" s="43" t="n">
         <v>2</v>
       </c>
       <c r="B3" s="35" t="inlineStr">
@@ -4736,7 +7690,7 @@
           <t>★★★☆☆ 同瘤种/同线数/同期别，但方案不对等（联合 vs 单药）</t>
         </is>
       </c>
-      <c r="D3" s="32" t="inlineStr">
+      <c r="D3" s="44" t="inlineStr">
         <is>
           <t>三阴性乳腺癌（TNBC）</t>
         </is>
@@ -4798,7 +7752,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="30" t="n">
+      <c r="A4" s="43" t="n">
         <v>3</v>
       </c>
       <c r="B4" s="35" t="inlineStr">
@@ -4811,7 +7765,7 @@
           <t>★★☆☆☆ 同瘤种/同线数/同方案（单药），但样本量差 20 倍</t>
         </is>
       </c>
-      <c r="D4" s="32" t="inlineStr">
+      <c r="D4" s="44" t="inlineStr">
         <is>
           <t>卵巢癌 / 输卵管 / 原发腹膜癌</t>
         </is>
@@ -4982,7 +7936,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="30" t="n">
+      <c r="A2" s="43" t="n">
         <v>1</v>
       </c>
       <c r="B2" s="19" t="inlineStr">
@@ -4995,7 +7949,7 @@
           <t>不符合筛选条件，但价值最高：K药 被头对头击败</t>
         </is>
       </c>
-      <c r="D2" s="32" t="inlineStr">
+      <c r="D2" s="44" t="inlineStr">
         <is>
           <t>NSCLC</t>
         </is>
@@ -5057,7 +8011,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="30" t="n">
+      <c r="A3" s="43" t="n">
         <v>2</v>
       </c>
       <c r="B3" s="19" t="inlineStr">
@@ -5070,7 +8024,7 @@
           <t>两者均成功，未头对头</t>
         </is>
       </c>
-      <c r="D3" s="32" t="inlineStr">
+      <c r="D3" s="44" t="inlineStr">
         <is>
           <t>NSCLC（鳞）</t>
         </is>
@@ -5132,7 +8086,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="30" t="n">
+      <c r="A4" s="43" t="n">
         <v>3</v>
       </c>
       <c r="B4" s="19" t="inlineStr">
@@ -5145,7 +8099,7 @@
           <t>两者均成功，对照强度差一个量级</t>
         </is>
       </c>
-      <c r="D4" s="32" t="inlineStr">
+      <c r="D4" s="44" t="inlineStr">
         <is>
           <t>胆道癌（BTC）</t>
         </is>
@@ -5207,7 +8161,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="30" t="n">
+      <c r="A5" s="43" t="n">
         <v>4</v>
       </c>
       <c r="B5" s="19" t="inlineStr">
@@ -5220,7 +8174,7 @@
           <t>K药 已 III 期成功，AK112 仅 II 期单臂</t>
         </is>
       </c>
-      <c r="D5" s="32" t="inlineStr">
+      <c r="D5" s="44" t="inlineStr">
         <is>
           <t>NSCLC</t>
         </is>
@@ -5282,7 +8236,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="30" t="n">
+      <c r="A6" s="43" t="n">
         <v>5</v>
       </c>
       <c r="B6" s="19" t="inlineStr">
@@ -5295,7 +8249,7 @@
           <t>K药 已 III 期成功，AK112 仅单中心 IIT</t>
         </is>
       </c>
-      <c r="D6" s="32" t="inlineStr">
+      <c r="D6" s="44" t="inlineStr">
         <is>
           <t>头颈鳞癌（HNSCC）</t>
         </is>
@@ -5357,7 +8311,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="30" t="n">
+      <c r="A7" s="43" t="n">
         <v>6</v>
       </c>
       <c r="B7" s="19" t="inlineStr">
@@ -5370,7 +8324,7 @@
           <t>K药 已 III 期成功，同期别 ORR 差距有限</t>
         </is>
       </c>
-      <c r="D7" s="32" t="inlineStr">
+      <c r="D7" s="44" t="inlineStr">
         <is>
           <t>胃 / 胃食管结合部腺癌</t>
         </is>
@@ -5541,7 +8495,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="30" t="n">
+      <c r="A2" s="43" t="n">
         <v>1</v>
       </c>
       <c r="B2" s="36" t="inlineStr">
@@ -5554,7 +8508,7 @@
           <t>K药 机制上不适用，不应计入战绩对比</t>
         </is>
       </c>
-      <c r="D2" s="32" t="inlineStr">
+      <c r="D2" s="44" t="inlineStr">
         <is>
           <t>NSCLC</t>
         </is>
@@ -5616,7 +8570,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="30" t="n">
+      <c r="A3" s="43" t="n">
         <v>2</v>
       </c>
       <c r="B3" s="36" t="inlineStr">
@@ -5629,7 +8583,7 @@
           <t>K药 明确失败，但 AK112 数据未公开，无法比较</t>
         </is>
       </c>
-      <c r="D3" s="32" t="inlineStr">
+      <c r="D3" s="44" t="inlineStr">
         <is>
           <t>胰腺癌（PDAC）</t>
         </is>
@@ -5691,7 +8645,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="30" t="n">
+      <c r="A4" s="43" t="n">
         <v>3</v>
       </c>
       <c r="B4" s="36" t="inlineStr">
@@ -5704,7 +8658,7 @@
           <t>期别相差三级，且 AK112 自己也未验证</t>
         </is>
       </c>
-      <c r="D4" s="32" t="inlineStr">
+      <c r="D4" s="44" t="inlineStr">
         <is>
           <t>小细胞肺癌（SCLC）</t>
         </is>
@@ -5766,7 +8720,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="30" t="n">
+      <c r="A5" s="43" t="n">
         <v>4</v>
       </c>
       <c r="B5" s="36" t="inlineStr">
@@ -5779,7 +8733,7 @@
           <t>方案不对等（联合 vs 单药），且 K药 最终在 III 期成功</t>
         </is>
       </c>
-      <c r="D5" s="32" t="inlineStr">
+      <c r="D5" s="44" t="inlineStr">
         <is>
           <t>胆道癌（BTC）</t>
         </is>
@@ -6349,7 +9303,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="30" t="n">
+      <c r="A2" s="43" t="n">
         <v>1</v>
       </c>
       <c r="B2" s="31" t="inlineStr">
@@ -6362,7 +9316,7 @@
           <t>★★★★★ 同瘤种/同线数/同期别/同方案（单药）</t>
         </is>
       </c>
-      <c r="D2" s="32" t="inlineStr">
+      <c r="D2" s="44" t="inlineStr">
         <is>
           <t>肝细胞癌（HCC）</t>
         </is>
@@ -6424,7 +9378,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="30" t="n">
+      <c r="A3" s="43" t="n">
         <v>2</v>
       </c>
       <c r="B3" s="31" t="inlineStr">
@@ -6437,7 +9391,7 @@
           <t>★★★★★ 同瘤种/同线数/同期别/同方案（单药）</t>
         </is>
       </c>
-      <c r="D3" s="32" t="inlineStr">
+      <c r="D3" s="44" t="inlineStr">
         <is>
           <t>宫颈癌</t>
         </is>
@@ -6499,7 +9453,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="30" t="n">
+      <c r="A4" s="43" t="n">
         <v>3</v>
       </c>
       <c r="B4" s="31" t="inlineStr">
@@ -6512,7 +9466,7 @@
           <t>★★★★☆ 同瘤种/同方案（单药），期别 II vs Ia/Ib+II</t>
         </is>
       </c>
-      <c r="D4" s="32" t="inlineStr">
+      <c r="D4" s="44" t="inlineStr">
         <is>
           <t>子宫内膜癌</t>
         </is>
@@ -6574,7 +9528,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="30" t="n">
+      <c r="A5" s="43" t="n">
         <v>4</v>
       </c>
       <c r="B5" s="31" t="inlineStr">
@@ -6587,7 +9541,7 @@
           <t>★★★☆☆ 同瘤种/同线数/同方案（单药），但 AK112 n=10 且剂量偏低</t>
         </is>
       </c>
-      <c r="D5" s="32" t="inlineStr">
+      <c r="D5" s="44" t="inlineStr">
         <is>
           <t>头颈鳞癌（HNSCC）</t>
         </is>
@@ -6649,7 +9603,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="30" t="n">
+      <c r="A6" s="43" t="n">
         <v>5</v>
       </c>
       <c r="B6" s="35" t="inlineStr">
@@ -6662,7 +9616,7 @@
           <t>★★★★☆ 同瘤种/同线数/同期别，且 K药 即为对照组</t>
         </is>
       </c>
-      <c r="D6" s="32" t="inlineStr">
+      <c r="D6" s="44" t="inlineStr">
         <is>
           <t>NSCLC（鳞）</t>
         </is>
@@ -6724,7 +9678,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="30" t="n">
+      <c r="A7" s="43" t="n">
         <v>6</v>
       </c>
       <c r="B7" s="36" t="inlineStr">
@@ -6737,7 +9691,7 @@
           <t>同瘤种/同线数/同期别/同方案 —— 但双方都失败</t>
         </is>
       </c>
-      <c r="D7" s="32" t="inlineStr">
+      <c r="D7" s="44" t="inlineStr">
         <is>
           <t>NSCLC（非鳞，EGFR 突变）</t>
         </is>
@@ -6799,7 +9753,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="30" t="n">
+      <c r="A8" s="43" t="n">
         <v>7</v>
       </c>
       <c r="B8" s="36" t="inlineStr">
@@ -6812,7 +9766,7 @@
           <t>同瘤种/同线数/同方案（单药）—— 双方均未获批</t>
         </is>
       </c>
-      <c r="D8" s="32" t="inlineStr">
+      <c r="D8" s="44" t="inlineStr">
         <is>
           <t>卵巢癌 / 输卵管 / 原发腹膜癌</t>
         </is>
@@ -6874,7 +9828,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="30" t="n">
+      <c r="A9" s="43" t="n">
         <v>8</v>
       </c>
       <c r="B9" s="36" t="inlineStr">
@@ -6887,7 +9841,7 @@
           <t>非疗效性失败，不可解读为阴性</t>
         </is>
       </c>
-      <c r="D9" s="32" t="inlineStr">
+      <c r="D9" s="44" t="inlineStr">
         <is>
           <t>卵巢癌</t>
         </is>
@@ -6949,7 +9903,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="30" t="n">
+      <c r="A10" s="43" t="n">
         <v>9</v>
       </c>
       <c r="B10" s="36" t="inlineStr">
@@ -6962,7 +9916,7 @@
           <t>同瘤种/同方案（单药）—— K药 更差</t>
         </is>
       </c>
-      <c r="D10" s="32" t="inlineStr">
+      <c r="D10" s="44" t="inlineStr">
         <is>
           <t>结直肠癌（MSS/pMMR）</t>
         </is>
@@ -7024,7 +9978,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="30" t="n">
+      <c r="A11" s="43" t="n">
         <v>10</v>
       </c>
       <c r="B11" s="36" t="inlineStr">
@@ -7037,7 +9991,7 @@
           <t>同瘤种/同方案（单药）—— K药 数据更完整但同样未获批</t>
         </is>
       </c>
-      <c r="D11" s="32" t="inlineStr">
+      <c r="D11" s="44" t="inlineStr">
         <is>
           <t>恶性胸膜间皮瘤</t>
         </is>
@@ -7099,7 +10053,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="30" t="n">
+      <c r="A12" s="43" t="n">
         <v>11</v>
       </c>
       <c r="B12" s="36" t="inlineStr">
@@ -7112,7 +10066,7 @@
           <t>同瘤种/同方案（单药）—— K药 数据更完整但同样未获批</t>
         </is>
       </c>
-      <c r="D12" s="32" t="inlineStr">
+      <c r="D12" s="44" t="inlineStr">
         <is>
           <t>肛管鳞癌</t>
         </is>

</xml_diff>